<commit_message>
Fix Unit 2 assignment: rebuild in single pass, strip orphaned SharePoint metadata causing Excel repair prompt
</commit_message>
<xml_diff>
--- a/Term_02/BUS 1102-01 Basic Accounting - AY2027-T1/Assignments/Unit2_Assignment.xlsx
+++ b/Term_02/BUS 1102-01 Basic Accounting - AY2027-T1/Assignments/Unit2_Assignment.xlsx
@@ -21,7 +21,7 @@
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -75,7 +75,6 @@
     <font>
       <b val="1"/>
     </font>
-    <font/>
     <font>
       <sz val="10"/>
     </font>
@@ -394,7 +393,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="104">
+  <cellXfs count="98">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -577,11 +576,6 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="2" fillId="2" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="2" fillId="2" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
@@ -591,22 +585,17 @@
     </xf>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="8" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="8" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="9" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1715,7 +1704,7 @@
           <t>Oct-01</t>
         </is>
       </c>
-      <c r="D3" s="87" t="n">
+      <c r="D3" s="84" t="n">
         <v>50000</v>
       </c>
       <c r="E3" s="56" t="inlineStr">
@@ -1723,7 +1712,7 @@
           <t>Oct-02</t>
         </is>
       </c>
-      <c r="F3" s="88" t="n">
+      <c r="F3" s="85" t="n">
         <v>5000</v>
       </c>
       <c r="K3" s="57" t="inlineStr">
@@ -1731,7 +1720,7 @@
           <t>Oct-05</t>
         </is>
       </c>
-      <c r="L3" s="88" t="n">
+      <c r="L3" s="85" t="n">
         <v>1500</v>
       </c>
       <c r="M3" s="58" t="n"/>
@@ -1743,7 +1732,7 @@
           <t>Oct-12</t>
         </is>
       </c>
-      <c r="D4" s="87" t="n">
+      <c r="D4" s="84" t="n">
         <v>4000</v>
       </c>
       <c r="E4" s="56" t="inlineStr">
@@ -1751,7 +1740,7 @@
           <t>Oct-03</t>
         </is>
       </c>
-      <c r="F4" s="89" t="n">
+      <c r="F4" s="86" t="n">
         <v>2000</v>
       </c>
       <c r="G4" s="42" t="n"/>
@@ -1762,7 +1751,7 @@
           <t>Balance</t>
         </is>
       </c>
-      <c r="L4" s="90" t="n">
+      <c r="L4" s="87" t="n">
         <v>1500</v>
       </c>
       <c r="M4" s="43" t="n"/>
@@ -1773,7 +1762,7 @@
           <t>Oct-25</t>
         </is>
       </c>
-      <c r="D5" s="87" t="n">
+      <c r="D5" s="84" t="n">
         <v>7500</v>
       </c>
       <c r="E5" s="56" t="inlineStr">
@@ -1781,7 +1770,7 @@
           <t>Oct-10</t>
         </is>
       </c>
-      <c r="F5" s="89" t="n">
+      <c r="F5" s="86" t="n">
         <v>1000</v>
       </c>
       <c r="G5" s="42" t="n"/>
@@ -1799,7 +1788,7 @@
           <t>Oct-15</t>
         </is>
       </c>
-      <c r="F6" s="89" t="n">
+      <c r="F6" s="86" t="n">
         <v>3500</v>
       </c>
       <c r="G6" s="42" t="n"/>
@@ -1815,7 +1804,7 @@
           <t>Oct-18</t>
         </is>
       </c>
-      <c r="F7" s="88" t="n">
+      <c r="F7" s="85" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -1828,7 +1817,7 @@
           <t>Oct-30</t>
         </is>
       </c>
-      <c r="F8" s="88" t="n">
+      <c r="F8" s="85" t="n">
         <v>3000</v>
       </c>
       <c r="K8" t="inlineStr">
@@ -1845,7 +1834,7 @@
           <t>Balance</t>
         </is>
       </c>
-      <c r="D9" s="88" t="n">
+      <c r="D9" s="85" t="n">
         <v>45000</v>
       </c>
       <c r="J9" s="47" t="n"/>
@@ -1869,7 +1858,7 @@
           <t>Oct-07</t>
         </is>
       </c>
-      <c r="L10" s="88" t="n">
+      <c r="L10" s="85" t="n">
         <v>6000</v>
       </c>
       <c r="M10" s="58" t="inlineStr">
@@ -1877,7 +1866,7 @@
           <t>Oct-12</t>
         </is>
       </c>
-      <c r="N10" s="88" t="n">
+      <c r="N10" s="85" t="n">
         <v>4000</v>
       </c>
     </row>
@@ -1891,7 +1880,7 @@
           <t>Balance</t>
         </is>
       </c>
-      <c r="L11" s="90" t="n">
+      <c r="L11" s="87" t="n">
         <v>2000</v>
       </c>
       <c r="M11" s="43" t="n"/>
@@ -1966,7 +1955,7 @@
           <t>Oct-01</t>
         </is>
       </c>
-      <c r="F19" s="88" t="n">
+      <c r="F19" s="85" t="n">
         <v>50000</v>
       </c>
       <c r="K19" s="46" t="n"/>
@@ -1976,7 +1965,7 @@
           <t>Oct-07</t>
         </is>
       </c>
-      <c r="N19" s="88" t="n">
+      <c r="N19" s="85" t="n">
         <v>6000</v>
       </c>
     </row>
@@ -1989,7 +1978,7 @@
           <t>Balance</t>
         </is>
       </c>
-      <c r="F20" s="90" t="n">
+      <c r="F20" s="87" t="n">
         <v>50000</v>
       </c>
       <c r="G20" s="43" t="n"/>
@@ -2000,7 +1989,7 @@
           <t>Oct-25</t>
         </is>
       </c>
-      <c r="N20" s="88" t="n">
+      <c r="N20" s="85" t="n">
         <v>7500</v>
       </c>
     </row>
@@ -2011,7 +2000,7 @@
           <t>Balance</t>
         </is>
       </c>
-      <c r="N21" s="88" t="n">
+      <c r="N21" s="85" t="n">
         <v>13500</v>
       </c>
     </row>
@@ -2087,7 +2076,7 @@
           <t>Oct-02</t>
         </is>
       </c>
-      <c r="D28" s="88" t="n">
+      <c r="D28" s="85" t="n">
         <v>10000</v>
       </c>
       <c r="E28" s="58" t="n"/>
@@ -2096,7 +2085,7 @@
           <t>Oct-15</t>
         </is>
       </c>
-      <c r="L28" s="87" t="n">
+      <c r="L28" s="84" t="n">
         <v>3500</v>
       </c>
       <c r="M28" s="56" t="n"/>
@@ -2107,7 +2096,7 @@
           <t>Oct-28</t>
         </is>
       </c>
-      <c r="D29" s="88" t="n">
+      <c r="D29" s="85" t="n">
         <v>1000</v>
       </c>
       <c r="E29" s="58" t="n"/>
@@ -2116,7 +2105,7 @@
           <t>Balance</t>
         </is>
       </c>
-      <c r="L29" s="87" t="n">
+      <c r="L29" s="84" t="n">
         <v>3500</v>
       </c>
       <c r="M29" s="56" t="n"/>
@@ -2201,7 +2190,7 @@
           <t>Oct-10</t>
         </is>
       </c>
-      <c r="D37" s="91" t="n">
+      <c r="D37" s="88" t="n">
         <v>1000</v>
       </c>
       <c r="E37" s="58" t="inlineStr">
@@ -2209,7 +2198,7 @@
           <t>Oct-02</t>
         </is>
       </c>
-      <c r="F37" s="88" t="n">
+      <c r="F37" s="85" t="n">
         <v>5000</v>
       </c>
       <c r="K37" s="57" t="inlineStr">
@@ -2217,7 +2206,7 @@
           <t>Oct-20</t>
         </is>
       </c>
-      <c r="L37" s="87" t="n">
+      <c r="L37" s="84" t="n">
         <v>1200</v>
       </c>
       <c r="M37" s="56" t="n"/>
@@ -2228,7 +2217,7 @@
           <t>Oct-30</t>
         </is>
       </c>
-      <c r="D38" s="91" t="n">
+      <c r="D38" s="88" t="n">
         <v>3000</v>
       </c>
       <c r="E38" s="58" t="inlineStr">
@@ -2236,7 +2225,7 @@
           <t>Oct-05</t>
         </is>
       </c>
-      <c r="F38" s="90" t="n">
+      <c r="F38" s="87" t="n">
         <v>1500</v>
       </c>
       <c r="G38" s="43" t="n"/>
@@ -2246,7 +2235,7 @@
           <t>Balance</t>
         </is>
       </c>
-      <c r="L38" s="87" t="n">
+      <c r="L38" s="84" t="n">
         <v>1200</v>
       </c>
       <c r="M38" s="56" t="n"/>
@@ -2259,7 +2248,7 @@
           <t>Oct-20</t>
         </is>
       </c>
-      <c r="F39" s="88" t="n">
+      <c r="F39" s="85" t="n">
         <v>1200</v>
       </c>
       <c r="K39" s="46" t="n"/>
@@ -2271,7 +2260,7 @@
           <t>Oct-28</t>
         </is>
       </c>
-      <c r="F40" s="88" t="n">
+      <c r="F40" s="85" t="n">
         <v>1000</v>
       </c>
       <c r="K40" s="56" t="n"/>
@@ -2284,7 +2273,7 @@
           <t>Balance</t>
         </is>
       </c>
-      <c r="F41" s="88" t="n">
+      <c r="F41" s="85" t="n">
         <v>4700</v>
       </c>
       <c r="G41" s="58" t="n"/>
@@ -2329,7 +2318,7 @@
           <t>Oct-03</t>
         </is>
       </c>
-      <c r="D46" s="91" t="n">
+      <c r="D46" s="88" t="n">
         <v>2000</v>
       </c>
       <c r="E46" s="58" t="n"/>
@@ -2341,7 +2330,7 @@
           <t>Balance</t>
         </is>
       </c>
-      <c r="D47" s="88" t="n">
+      <c r="D47" s="85" t="n">
         <v>2000</v>
       </c>
       <c r="E47" s="43" t="n"/>
@@ -2593,7 +2582,7 @@
           <t>Oct-18</t>
         </is>
       </c>
-      <c r="D77" s="88" t="n">
+      <c r="D77" s="85" t="n">
         <v>2000</v>
       </c>
       <c r="K77" s="50" t="n"/>
@@ -2605,7 +2594,7 @@
           <t>Balance</t>
         </is>
       </c>
-      <c r="D78" s="90" t="n">
+      <c r="D78" s="87" t="n">
         <v>2000</v>
       </c>
       <c r="E78" s="43" t="n"/>
@@ -2647,13 +2636,13 @@
   </cols>
   <sheetData>
     <row r="1" ht="14.45" customHeight="1">
-      <c r="A1" s="84" t="inlineStr">
+      <c r="A1" s="89" t="inlineStr">
         <is>
           <t>Trial Balance Urban Path Co.</t>
         </is>
       </c>
-      <c r="B1" s="85" t="n"/>
-      <c r="C1" s="86" t="n"/>
+      <c r="B1" s="90" t="n"/>
+      <c r="C1" s="91" t="n"/>
     </row>
     <row r="2" ht="14.45" customHeight="1">
       <c r="A2" s="31" t="inlineStr">
@@ -2817,77 +2806,48 @@
       <c r="C16" s="32" t="n"/>
     </row>
     <row r="17" ht="14.45" customHeight="1">
-      <c r="A17" s="98" t="n"/>
-      <c r="B17" s="98" t="n"/>
-      <c r="C17" s="99" t="n"/>
-      <c r="D17" s="100" t="n"/>
-      <c r="E17" s="100" t="n"/>
-      <c r="F17" s="100" t="n"/>
-      <c r="G17" s="100" t="n"/>
-      <c r="H17" s="100" t="n"/>
-      <c r="I17" s="100" t="n"/>
-      <c r="J17" s="100" t="n"/>
-      <c r="K17" s="100" t="n"/>
-      <c r="L17" s="100" t="n"/>
-      <c r="M17" s="100" t="n"/>
-      <c r="N17" s="100" t="n"/>
-    </row>
-    <row r="18" ht="90" customHeight="1">
-      <c r="A18" s="101" t="n"/>
+      <c r="A17" s="30" t="n"/>
+      <c r="B17" s="30" t="n"/>
+      <c r="C17" s="32" t="n"/>
+    </row>
+    <row r="18" ht="14.45" customHeight="1">
+      <c r="A18" s="30" t="n"/>
+      <c r="B18" s="30" t="n"/>
+      <c r="C18" s="32" t="n"/>
     </row>
     <row r="19" ht="14.45" customHeight="1">
-      <c r="A19" s="98" t="n"/>
-      <c r="B19" s="102" t="n"/>
-      <c r="C19" s="99" t="n"/>
-      <c r="D19" s="100" t="n"/>
-      <c r="E19" s="100" t="n"/>
-      <c r="F19" s="100" t="n"/>
-      <c r="G19" s="100" t="n"/>
-      <c r="H19" s="100" t="n"/>
-      <c r="I19" s="100" t="n"/>
-      <c r="J19" s="100" t="n"/>
-      <c r="K19" s="100" t="n"/>
-      <c r="L19" s="100" t="n"/>
-      <c r="M19" s="100" t="n"/>
-      <c r="N19" s="100" t="n"/>
+      <c r="A19" s="30" t="n"/>
+      <c r="B19" s="35" t="n"/>
+      <c r="C19" s="32" t="n"/>
     </row>
     <row r="20" ht="14.45" customHeight="1">
-      <c r="A20" s="98" t="n"/>
-      <c r="B20" s="98" t="n"/>
-      <c r="C20" s="99" t="n"/>
-      <c r="D20" s="100" t="n"/>
-      <c r="E20" s="100" t="n"/>
-      <c r="F20" s="100" t="n"/>
-      <c r="G20" s="100" t="n"/>
-      <c r="H20" s="100" t="n"/>
-      <c r="I20" s="100" t="n"/>
-      <c r="J20" s="100" t="n"/>
-      <c r="K20" s="100" t="n"/>
-      <c r="L20" s="100" t="n"/>
-      <c r="M20" s="100" t="n"/>
-      <c r="N20" s="100" t="n"/>
-    </row>
-    <row r="21" ht="45" customHeight="1">
-      <c r="A21" s="98" t="n"/>
+      <c r="A20" s="30" t="n"/>
+      <c r="B20" s="30" t="n"/>
+      <c r="C20" s="32" t="n"/>
+    </row>
+    <row r="21" ht="14.45" customHeight="1">
+      <c r="A21" s="30" t="n"/>
+      <c r="B21" s="35" t="n"/>
+      <c r="C21" s="32" t="n"/>
     </row>
     <row r="22" ht="14.45" customHeight="1">
       <c r="A22" s="34" t="n"/>
       <c r="B22" s="36" t="n"/>
       <c r="C22" s="38" t="n"/>
     </row>
-    <row r="25" ht="30" customHeight="1">
-      <c r="A25" s="103" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="97" t="inlineStr">
         <is>
           <t>Journal entries are the accounting cycle's starting point: every transaction is first recorded chronologically in a journal, in debit-and-credit form, before it touches any other record (Franklin et al., 2022). Ledgers, organized as T-accounts, then sort each entry into its own account so a business can see a running balance for cash, revenue, or any other item. That organized ledger data is what makes an accurate trial balance possible, since a trial balance simply lists every ledger balance to confirm total debits equal total credits before financial statements get prepared (Franklin et al., 2022).
-Reference: Franklin, M., Graybeal, P., Cooper, D., Bean, L., Burt, I., Carr, S., Collins, D. T., Coram, S., Creech, K., Czyzewski, A., Gauci, M., Greenman, C., Haselkorn, M., Irujo, C., Johnson, C., Khanlarian, C., Lukshaitis, T., Luna, D., Nantz, B., … Woolley, D. (2022). Principles of accounting, volume 1: Financial accounting. OpenStax. Licensed under CC 4.0. https://openstax.org/details/books/principles-financial-accounting</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="30" customHeight="1"/>
-    <row r="27" ht="30" customHeight="1"/>
-    <row r="28" ht="30" customHeight="1"/>
-    <row r="29" ht="30" customHeight="1"/>
-    <row r="30" ht="30" customHeight="1"/>
+Reference: Franklin, M., Graybeal, P., Cooper, D., Bean, L., Burt, I., Carr, S., Collins, D. T., Coram, S., Creech, K., Czyzewski, A., Gauci, M., Greenman, C., Haselkorn, M., Irujo, C., Johnson, C., Khanlarian, C., Lukshaitis, T., Luna, D., Nantz, B, ... Woolley, D. (2022). Principles of accounting, volume 1: Financial accounting. OpenStax. Licensed under CC 4.0. https://openstax.org/details/books/principles-financial-accounting</t>
+        </is>
+      </c>
+    </row>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:C1"/>

</xml_diff>

<commit_message>
Restore T-account box borders lost in xlsxwriter rebuild
</commit_message>
<xml_diff>
--- a/Term_02/BUS 1102-01 Basic Accounting - AY2027-T1/Assignments/Unit2_Assignment.xlsx
+++ b/Term_02/BUS 1102-01 Basic Accounting - AY2027-T1/Assignments/Unit2_Assignment.xlsx
@@ -249,7 +249,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -272,19 +272,151 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -605,334 +737,334 @@
       <c r="B3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="2"/>
+      <c r="D3" s="3"/>
       <c r="E3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="4" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="4" spans="2:6">
-      <c r="B4" t="s">
+      <c r="B4" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="E4" s="3">
+      <c r="E4" s="7">
         <v>50000</v>
       </c>
     </row>
     <row r="5" spans="2:6">
-      <c r="C5" t="s">
+      <c r="C5" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="F5" s="3">
+      <c r="F5" s="9">
         <v>50000</v>
       </c>
     </row>
     <row r="6" spans="2:6">
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="10" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="7" spans="2:6">
-      <c r="B7" t="s">
+      <c r="B7" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="E7" s="3">
+      <c r="E7" s="12">
         <v>10000</v>
       </c>
     </row>
     <row r="8" spans="2:6">
-      <c r="C8" t="s">
+      <c r="C8" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="F8" s="3">
+      <c r="F8" s="9">
         <v>5000</v>
       </c>
     </row>
     <row r="9" spans="2:6">
-      <c r="C9" t="s">
+      <c r="C9" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="F9" s="3">
+      <c r="F9" s="9">
         <v>5000</v>
       </c>
     </row>
     <row r="10" spans="2:6">
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="13" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="11" spans="2:6">
-      <c r="B11" t="s">
+      <c r="B11" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="E11" s="3">
+      <c r="E11" s="12">
         <v>2000</v>
       </c>
     </row>
     <row r="12" spans="2:6">
-      <c r="C12" t="s">
+      <c r="C12" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="F12" s="3">
+      <c r="F12" s="15">
         <v>2000</v>
       </c>
     </row>
     <row r="13" spans="2:6">
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="16" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="14" spans="2:6">
-      <c r="B14" t="s">
+      <c r="B14" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="E14" s="3">
+      <c r="E14" s="12">
         <v>1500</v>
       </c>
     </row>
     <row r="15" spans="2:6">
-      <c r="C15" t="s">
+      <c r="C15" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="F15" s="3">
+      <c r="F15" s="9">
         <v>1500</v>
       </c>
     </row>
     <row r="16" spans="2:6">
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="13" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="17" spans="2:6">
-      <c r="B17" t="s">
+      <c r="B17" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="E17" s="3">
+      <c r="E17" s="12">
         <v>6000</v>
       </c>
     </row>
     <row r="18" spans="2:6">
-      <c r="C18" t="s">
+      <c r="C18" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="F18" s="3">
+      <c r="F18" s="15">
         <v>6000</v>
       </c>
     </row>
     <row r="19" spans="2:6">
-      <c r="C19" s="4" t="s">
+      <c r="C19" s="16" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="20" spans="2:6">
-      <c r="B20" t="s">
+      <c r="B20" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C20" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="E20" s="3">
+      <c r="E20" s="12">
         <v>1000</v>
       </c>
     </row>
     <row r="21" spans="2:6">
-      <c r="C21" t="s">
+      <c r="C21" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="F21" s="3">
+      <c r="F21" s="9">
         <v>1000</v>
       </c>
     </row>
     <row r="22" spans="2:6">
-      <c r="C22" s="4" t="s">
+      <c r="C22" s="13" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="23" spans="2:6">
-      <c r="B23" t="s">
+      <c r="B23" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C23" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="E23" s="3">
+      <c r="E23" s="12">
         <v>4000</v>
       </c>
     </row>
     <row r="24" spans="2:6">
-      <c r="C24" t="s">
+      <c r="C24" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="F24" s="3">
+      <c r="F24" s="15">
         <v>4000</v>
       </c>
     </row>
     <row r="25" spans="2:6">
-      <c r="C25" s="4" t="s">
+      <c r="C25" s="16" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="26" spans="2:6">
-      <c r="B26" t="s">
+      <c r="B26" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C26" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="E26" s="3">
+      <c r="E26" s="12">
         <v>3500</v>
       </c>
     </row>
     <row r="27" spans="2:6">
-      <c r="C27" t="s">
+      <c r="C27" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="F27" s="3">
+      <c r="F27" s="9">
         <v>3500</v>
       </c>
     </row>
     <row r="28" spans="2:6">
-      <c r="C28" s="4" t="s">
+      <c r="C28" s="13" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="29" spans="2:6">
-      <c r="B29" t="s">
+      <c r="B29" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="C29" t="s">
+      <c r="C29" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="E29" s="3">
+      <c r="E29" s="12">
         <v>2000</v>
       </c>
     </row>
     <row r="30" spans="2:6">
-      <c r="C30" t="s">
+      <c r="C30" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="F30" s="3">
+      <c r="F30" s="15">
         <v>2000</v>
       </c>
     </row>
     <row r="31" spans="2:6">
-      <c r="C31" s="4" t="s">
+      <c r="C31" s="16" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="32" spans="2:6">
-      <c r="B32" t="s">
+      <c r="B32" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="C32" t="s">
+      <c r="C32" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="E32" s="3">
+      <c r="E32" s="12">
         <v>1200</v>
       </c>
     </row>
     <row r="33" spans="2:6">
-      <c r="C33" t="s">
+      <c r="C33" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="F33" s="3">
+      <c r="F33" s="9">
         <v>1200</v>
       </c>
     </row>
     <row r="34" spans="2:6">
-      <c r="C34" s="4" t="s">
+      <c r="C34" s="13" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="35" spans="2:6">
-      <c r="B35" t="s">
+      <c r="B35" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="C35" t="s">
+      <c r="C35" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="E35" s="3">
+      <c r="E35" s="12">
         <v>7500</v>
       </c>
     </row>
     <row r="36" spans="2:6">
-      <c r="C36" t="s">
+      <c r="C36" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="F36" s="3">
+      <c r="F36" s="15">
         <v>7500</v>
       </c>
     </row>
     <row r="37" spans="2:6">
-      <c r="C37" s="4" t="s">
+      <c r="C37" s="16" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="38" spans="2:6">
-      <c r="B38" t="s">
+      <c r="B38" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="C38" t="s">
+      <c r="C38" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="E38" s="3">
+      <c r="E38" s="12">
         <v>1000</v>
       </c>
     </row>
     <row r="39" spans="2:6">
-      <c r="C39" t="s">
+      <c r="C39" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="F39" s="3">
+      <c r="F39" s="9">
         <v>1000</v>
       </c>
     </row>
     <row r="40" spans="2:6">
-      <c r="C40" s="4" t="s">
+      <c r="C40" s="13" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="41" spans="2:6">
-      <c r="B41" t="s">
+      <c r="B41" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="C41" t="s">
+      <c r="C41" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="E41" s="3">
+      <c r="E41" s="12">
         <v>3000</v>
       </c>
     </row>
     <row r="42" spans="2:6">
-      <c r="C42" t="s">
+      <c r="C42" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="F42" s="3">
+      <c r="F42" s="15">
         <v>3000</v>
       </c>
     </row>
     <row r="43" spans="2:6">
-      <c r="C43" s="4" t="s">
+      <c r="C43" s="16" t="s">
         <v>44</v>
       </c>
     </row>
@@ -963,401 +1095,401 @@
   </cols>
   <sheetData>
     <row r="1" spans="3:14">
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="K1" s="18" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="2" spans="3:14">
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="K2" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="M2" s="2" t="s">
+      <c r="M2" s="20" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="3" spans="3:14">
-      <c r="C3" t="s">
+      <c r="C3" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="3">
+      <c r="D3" s="22">
         <v>50000</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F3" s="3">
+      <c r="F3" s="22">
         <v>5000</v>
       </c>
-      <c r="K3" t="s">
+      <c r="K3" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="L3" s="3">
+      <c r="L3" s="22">
         <v>1500</v>
       </c>
     </row>
     <row r="4" spans="3:14">
-      <c r="C4" t="s">
+      <c r="C4" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="22">
         <v>4000</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="F4" s="3">
+      <c r="F4" s="22">
         <v>2000</v>
       </c>
-      <c r="K4" s="6" t="s">
+      <c r="K4" s="24" t="s">
         <v>46</v>
       </c>
-      <c r="L4" s="7">
+      <c r="L4" s="25">
         <v>1500</v>
       </c>
     </row>
     <row r="5" spans="3:14">
-      <c r="C5" t="s">
+      <c r="C5" s="23" t="s">
         <v>39</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D5" s="22">
         <v>7500</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="F5" s="3">
+      <c r="F5" s="22">
         <v>1000</v>
       </c>
     </row>
     <row r="6" spans="3:14">
-      <c r="E6" t="s">
+      <c r="E6" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="F6" s="3">
+      <c r="F6" s="22">
         <v>3500</v>
       </c>
     </row>
     <row r="7" spans="3:14">
-      <c r="E7" t="s">
+      <c r="E7" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="F7" s="3">
+      <c r="F7" s="22">
         <v>2000</v>
       </c>
     </row>
     <row r="8" spans="3:14">
-      <c r="E8" t="s">
+      <c r="E8" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="F8" s="3">
+      <c r="F8" s="22">
         <v>3000</v>
       </c>
-      <c r="K8" s="5" t="s">
+      <c r="K8" s="18" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="9" spans="3:14">
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="24" t="s">
         <v>46</v>
       </c>
-      <c r="D9" s="7">
+      <c r="D9" s="25">
         <v>45000</v>
       </c>
-      <c r="K9" s="2" t="s">
+      <c r="K9" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="M9" s="2" t="s">
+      <c r="M9" s="20" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="10" spans="3:14">
-      <c r="K10" t="s">
+      <c r="K10" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="L10" s="3">
+      <c r="L10" s="22">
         <v>6000</v>
       </c>
-      <c r="M10" t="s">
+      <c r="M10" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="N10" s="3">
+      <c r="N10" s="22">
         <v>4000</v>
       </c>
     </row>
     <row r="11" spans="3:14">
-      <c r="K11" s="6" t="s">
+      <c r="K11" s="24" t="s">
         <v>46</v>
       </c>
-      <c r="L11" s="7">
+      <c r="L11" s="25">
         <v>2000</v>
       </c>
     </row>
     <row r="17" spans="3:14">
-      <c r="C17" s="5" t="s">
+      <c r="C17" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="K17" s="5" t="s">
+      <c r="K17" s="18" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="18" spans="3:14">
-      <c r="C18" s="2" t="s">
+      <c r="C18" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="E18" s="2" t="s">
+      <c r="E18" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="K18" s="2" t="s">
+      <c r="K18" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="M18" s="2" t="s">
+      <c r="M18" s="20" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="19" spans="3:14">
-      <c r="E19" t="s">
+      <c r="E19" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="F19" s="3">
+      <c r="F19" s="22">
         <v>50000</v>
       </c>
-      <c r="M19" t="s">
+      <c r="M19" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="N19" s="3">
+      <c r="N19" s="22">
         <v>6000</v>
       </c>
     </row>
     <row r="20" spans="3:14">
-      <c r="E20" s="6" t="s">
+      <c r="E20" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="F20" s="7">
+      <c r="F20" s="25">
         <v>50000</v>
       </c>
-      <c r="M20" t="s">
+      <c r="M20" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="N20" s="3">
+      <c r="N20" s="22">
         <v>7500</v>
       </c>
     </row>
     <row r="21" spans="3:14">
-      <c r="M21" s="6" t="s">
+      <c r="M21" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="N21" s="7">
+      <c r="N21" s="25">
         <v>13500</v>
       </c>
     </row>
     <row r="26" spans="3:14">
-      <c r="C26" s="5" t="s">
+      <c r="C26" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="K26" s="5" t="s">
+      <c r="K26" s="18" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="27" spans="3:14">
-      <c r="C27" s="2" t="s">
+      <c r="C27" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="E27" s="2" t="s">
+      <c r="E27" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="K27" s="2" t="s">
+      <c r="K27" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="M27" s="2" t="s">
+      <c r="M27" s="20" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="28" spans="3:14">
-      <c r="C28" t="s">
+      <c r="C28" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="D28" s="3">
+      <c r="D28" s="22">
         <v>10000</v>
       </c>
-      <c r="K28" t="s">
+      <c r="K28" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="L28" s="3">
+      <c r="L28" s="22">
         <v>3500</v>
       </c>
     </row>
     <row r="29" spans="3:14">
-      <c r="C29" t="s">
+      <c r="C29" s="23" t="s">
         <v>41</v>
       </c>
-      <c r="D29" s="3">
+      <c r="D29" s="22">
         <v>1000</v>
       </c>
-      <c r="K29" s="6" t="s">
+      <c r="K29" s="24" t="s">
         <v>46</v>
       </c>
-      <c r="L29" s="7">
+      <c r="L29" s="25">
         <v>3500</v>
       </c>
     </row>
     <row r="33" spans="2:13">
-      <c r="B33" s="6" t="s">
+      <c r="B33" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="C33" s="7">
+      <c r="C33" s="25">
         <v>11000</v>
       </c>
     </row>
     <row r="35" spans="2:13">
-      <c r="C35" s="5" t="s">
+      <c r="C35" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="K35" s="5" t="s">
+      <c r="K35" s="18" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="36" spans="2:13">
-      <c r="C36" s="2" t="s">
+      <c r="C36" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="E36" s="2" t="s">
+      <c r="E36" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="K36" s="2" t="s">
+      <c r="K36" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="M36" s="2" t="s">
+      <c r="M36" s="20" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="37" spans="2:13">
-      <c r="C37" t="s">
+      <c r="C37" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="D37" s="3">
+      <c r="D37" s="27">
         <v>1000</v>
       </c>
-      <c r="E37" t="s">
+      <c r="E37" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F37" s="3">
+      <c r="F37" s="22">
         <v>5000</v>
       </c>
-      <c r="K37" t="s">
+      <c r="K37" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="L37" s="3">
+      <c r="L37" s="22">
         <v>1200</v>
       </c>
     </row>
     <row r="38" spans="2:13">
-      <c r="C38" t="s">
+      <c r="C38" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="D38" s="3">
+      <c r="D38" s="27">
         <v>3000</v>
       </c>
-      <c r="E38" t="s">
+      <c r="E38" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="F38" s="3">
+      <c r="F38" s="22">
         <v>1500</v>
       </c>
-      <c r="K38" s="6" t="s">
+      <c r="K38" s="24" t="s">
         <v>46</v>
       </c>
-      <c r="L38" s="7">
+      <c r="L38" s="25">
         <v>1200</v>
       </c>
     </row>
     <row r="39" spans="2:13">
-      <c r="E39" t="s">
+      <c r="E39" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="F39" s="3">
+      <c r="F39" s="22">
         <v>1200</v>
       </c>
     </row>
     <row r="40" spans="2:13">
-      <c r="E40" t="s">
+      <c r="E40" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="F40" s="3">
+      <c r="F40" s="22">
         <v>1000</v>
       </c>
     </row>
     <row r="41" spans="2:13">
-      <c r="E41" s="6" t="s">
+      <c r="E41" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="F41" s="7">
+      <c r="F41" s="25">
         <v>4700</v>
       </c>
     </row>
     <row r="44" spans="2:13">
-      <c r="C44" s="5" t="s">
+      <c r="C44" s="18" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="45" spans="2:13">
-      <c r="C45" s="2" t="s">
+      <c r="C45" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="E45" s="2" t="s">
+      <c r="E45" s="20" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="46" spans="2:13">
-      <c r="C46" t="s">
+      <c r="C46" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="D46" s="3">
+      <c r="D46" s="27">
         <v>2000</v>
       </c>
     </row>
     <row r="47" spans="2:13">
-      <c r="C47" s="6" t="s">
+      <c r="C47" s="24" t="s">
         <v>46</v>
       </c>
-      <c r="D47" s="7">
+      <c r="D47" s="25">
         <v>2000</v>
       </c>
     </row>
     <row r="75" spans="3:5">
-      <c r="C75" s="5" t="s">
+      <c r="C75" s="18" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="76" spans="3:5">
-      <c r="C76" s="2" t="s">
+      <c r="C76" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="E76" s="2" t="s">
+      <c r="E76" s="20" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="77" spans="3:5">
-      <c r="C77" t="s">
+      <c r="C77" s="21" t="s">
         <v>33</v>
       </c>
-      <c r="D77" s="3">
+      <c r="D77" s="22">
         <v>2000</v>
       </c>
     </row>
     <row r="78" spans="3:5">
-      <c r="C78" s="6" t="s">
+      <c r="C78" s="24" t="s">
         <v>46</v>
       </c>
-      <c r="D78" s="7">
+      <c r="D78" s="25">
         <v>2000</v>
       </c>
     </row>
@@ -1368,232 +1500,232 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N21"/>
+  <dimension ref="A1:N22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="28.7109375" customWidth="1"/>
     <col min="2" max="3" width="15.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>52</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
-    <row r="2" spans="1:14">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:3">
+      <c r="A2" s="28" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="28" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="29" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:14">
-      <c r="A3" t="s">
+    <row r="3" spans="1:3">
+      <c r="A3" s="30" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="27">
         <v>45000</v>
       </c>
     </row>
-    <row r="4" spans="1:14">
-      <c r="A4" t="s">
+    <row r="4" spans="1:3">
+      <c r="A4" s="30" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="27">
         <v>2000</v>
       </c>
     </row>
-    <row r="5" spans="1:14">
-      <c r="A5" t="s">
+    <row r="5" spans="1:3">
+      <c r="A5" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="3">
+      <c r="B5" s="27">
         <v>1500</v>
       </c>
     </row>
-    <row r="6" spans="1:14">
-      <c r="A6" t="s">
+    <row r="6" spans="1:3">
+      <c r="A6" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="3">
+      <c r="B6" s="27">
         <v>11000</v>
       </c>
     </row>
-    <row r="7" spans="1:14">
-      <c r="A7" t="s">
+    <row r="7" spans="1:3">
+      <c r="A7" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="3">
+      <c r="C7" s="12">
         <v>4700</v>
       </c>
     </row>
-    <row r="8" spans="1:14">
-      <c r="A8" t="s">
+    <row r="8" spans="1:3">
+      <c r="A8" s="30" t="s">
         <v>53</v>
       </c>
-      <c r="C8" s="3">
+      <c r="C8" s="12">
         <v>50000</v>
       </c>
     </row>
-    <row r="9" spans="1:14">
-      <c r="A9" t="s">
+    <row r="9" spans="1:3">
+      <c r="A9" s="30" t="s">
         <v>34</v>
       </c>
-      <c r="B9" s="3">
+      <c r="B9" s="27">
         <v>2000</v>
       </c>
     </row>
-    <row r="10" spans="1:14">
-      <c r="A10" t="s">
+    <row r="10" spans="1:3">
+      <c r="A10" s="30" t="s">
         <v>49</v>
       </c>
-      <c r="C10" s="3">
+      <c r="C10" s="12">
         <v>13500</v>
       </c>
     </row>
-    <row r="11" spans="1:14">
-      <c r="A11" t="s">
+    <row r="11" spans="1:3">
+      <c r="A11" s="30" t="s">
         <v>31</v>
       </c>
-      <c r="B11" s="3">
+      <c r="B11" s="27">
         <v>3500</v>
       </c>
     </row>
-    <row r="12" spans="1:14">
-      <c r="A12" t="s">
+    <row r="12" spans="1:3">
+      <c r="A12" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="3">
+      <c r="B12" s="27">
         <v>2000</v>
       </c>
     </row>
-    <row r="13" spans="1:14">
-      <c r="A13" t="s">
+    <row r="13" spans="1:3">
+      <c r="A13" s="30" t="s">
         <v>37</v>
       </c>
-      <c r="B13" s="3">
+      <c r="B13" s="27">
         <v>1200</v>
       </c>
     </row>
-    <row r="14" spans="1:14">
-      <c r="A14" s="6" t="s">
+    <row r="14" spans="1:3">
+      <c r="A14" s="31" t="s">
         <v>54</v>
       </c>
-      <c r="B14" s="7">
+      <c r="B14" s="32">
         <v>68200</v>
       </c>
-      <c r="C14" s="7">
+      <c r="C14" s="33">
         <v>68200</v>
       </c>
     </row>
-    <row r="16" spans="1:14" ht="30" customHeight="1">
-      <c r="A16" s="8" t="s">
+    <row r="17" spans="1:14" ht="30" customHeight="1">
+      <c r="A17" s="34" t="s">
         <v>55</v>
       </c>
-      <c r="B16" s="8"/>
-      <c r="C16" s="8"/>
-      <c r="D16" s="8"/>
-      <c r="E16" s="8"/>
-      <c r="F16" s="8"/>
-      <c r="G16" s="8"/>
-      <c r="H16" s="8"/>
-      <c r="I16" s="8"/>
-      <c r="J16" s="8"/>
-      <c r="K16" s="8"/>
-      <c r="L16" s="8"/>
-      <c r="M16" s="8"/>
-      <c r="N16" s="8"/>
-    </row>
-    <row r="17" spans="1:14">
-      <c r="A17" s="8"/>
-      <c r="B17" s="8"/>
-      <c r="C17" s="8"/>
-      <c r="D17" s="8"/>
-      <c r="E17" s="8"/>
-      <c r="F17" s="8"/>
-      <c r="G17" s="8"/>
-      <c r="H17" s="8"/>
-      <c r="I17" s="8"/>
-      <c r="J17" s="8"/>
-      <c r="K17" s="8"/>
-      <c r="L17" s="8"/>
-      <c r="M17" s="8"/>
-      <c r="N17" s="8"/>
+      <c r="B17" s="34"/>
+      <c r="C17" s="34"/>
+      <c r="D17" s="34"/>
+      <c r="E17" s="34"/>
+      <c r="F17" s="34"/>
+      <c r="G17" s="34"/>
+      <c r="H17" s="34"/>
+      <c r="I17" s="34"/>
+      <c r="J17" s="34"/>
+      <c r="K17" s="34"/>
+      <c r="L17" s="34"/>
+      <c r="M17" s="34"/>
+      <c r="N17" s="34"/>
     </row>
     <row r="18" spans="1:14">
-      <c r="A18" s="8"/>
-      <c r="B18" s="8"/>
-      <c r="C18" s="8"/>
-      <c r="D18" s="8"/>
-      <c r="E18" s="8"/>
-      <c r="F18" s="8"/>
-      <c r="G18" s="8"/>
-      <c r="H18" s="8"/>
-      <c r="I18" s="8"/>
-      <c r="J18" s="8"/>
-      <c r="K18" s="8"/>
-      <c r="L18" s="8"/>
-      <c r="M18" s="8"/>
-      <c r="N18" s="8"/>
+      <c r="A18" s="34"/>
+      <c r="B18" s="34"/>
+      <c r="C18" s="34"/>
+      <c r="D18" s="34"/>
+      <c r="E18" s="34"/>
+      <c r="F18" s="34"/>
+      <c r="G18" s="34"/>
+      <c r="H18" s="34"/>
+      <c r="I18" s="34"/>
+      <c r="J18" s="34"/>
+      <c r="K18" s="34"/>
+      <c r="L18" s="34"/>
+      <c r="M18" s="34"/>
+      <c r="N18" s="34"/>
     </row>
     <row r="19" spans="1:14">
-      <c r="A19" s="8"/>
-      <c r="B19" s="8"/>
-      <c r="C19" s="8"/>
-      <c r="D19" s="8"/>
-      <c r="E19" s="8"/>
-      <c r="F19" s="8"/>
-      <c r="G19" s="8"/>
-      <c r="H19" s="8"/>
-      <c r="I19" s="8"/>
-      <c r="J19" s="8"/>
-      <c r="K19" s="8"/>
-      <c r="L19" s="8"/>
-      <c r="M19" s="8"/>
-      <c r="N19" s="8"/>
+      <c r="A19" s="34"/>
+      <c r="B19" s="34"/>
+      <c r="C19" s="34"/>
+      <c r="D19" s="34"/>
+      <c r="E19" s="34"/>
+      <c r="F19" s="34"/>
+      <c r="G19" s="34"/>
+      <c r="H19" s="34"/>
+      <c r="I19" s="34"/>
+      <c r="J19" s="34"/>
+      <c r="K19" s="34"/>
+      <c r="L19" s="34"/>
+      <c r="M19" s="34"/>
+      <c r="N19" s="34"/>
     </row>
     <row r="20" spans="1:14">
-      <c r="A20" s="8"/>
-      <c r="B20" s="8"/>
-      <c r="C20" s="8"/>
-      <c r="D20" s="8"/>
-      <c r="E20" s="8"/>
-      <c r="F20" s="8"/>
-      <c r="G20" s="8"/>
-      <c r="H20" s="8"/>
-      <c r="I20" s="8"/>
-      <c r="J20" s="8"/>
-      <c r="K20" s="8"/>
-      <c r="L20" s="8"/>
-      <c r="M20" s="8"/>
-      <c r="N20" s="8"/>
+      <c r="A20" s="34"/>
+      <c r="B20" s="34"/>
+      <c r="C20" s="34"/>
+      <c r="D20" s="34"/>
+      <c r="E20" s="34"/>
+      <c r="F20" s="34"/>
+      <c r="G20" s="34"/>
+      <c r="H20" s="34"/>
+      <c r="I20" s="34"/>
+      <c r="J20" s="34"/>
+      <c r="K20" s="34"/>
+      <c r="L20" s="34"/>
+      <c r="M20" s="34"/>
+      <c r="N20" s="34"/>
     </row>
     <row r="21" spans="1:14">
-      <c r="A21" s="8"/>
-      <c r="B21" s="8"/>
-      <c r="C21" s="8"/>
-      <c r="D21" s="8"/>
-      <c r="E21" s="8"/>
-      <c r="F21" s="8"/>
-      <c r="G21" s="8"/>
-      <c r="H21" s="8"/>
-      <c r="I21" s="8"/>
-      <c r="J21" s="8"/>
-      <c r="K21" s="8"/>
-      <c r="L21" s="8"/>
-      <c r="M21" s="8"/>
-      <c r="N21" s="8"/>
+      <c r="A21" s="34"/>
+      <c r="B21" s="34"/>
+      <c r="C21" s="34"/>
+      <c r="D21" s="34"/>
+      <c r="E21" s="34"/>
+      <c r="F21" s="34"/>
+      <c r="G21" s="34"/>
+      <c r="H21" s="34"/>
+      <c r="I21" s="34"/>
+      <c r="J21" s="34"/>
+      <c r="K21" s="34"/>
+      <c r="L21" s="34"/>
+      <c r="M21" s="34"/>
+      <c r="N21" s="34"/>
+    </row>
+    <row r="22" spans="1:14">
+      <c r="A22" s="34"/>
+      <c r="B22" s="34"/>
+      <c r="C22" s="34"/>
+      <c r="D22" s="34"/>
+      <c r="E22" s="34"/>
+      <c r="F22" s="34"/>
+      <c r="G22" s="34"/>
+      <c r="H22" s="34"/>
+      <c r="I22" s="34"/>
+      <c r="J22" s="34"/>
+      <c r="K22" s="34"/>
+      <c r="L22" s="34"/>
+      <c r="M22" s="34"/>
+      <c r="N22" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A16:N21"/>
+    <mergeCell ref="A17:N22"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix Unit 2 reference: APA italics, clickable URL, correct ellipsis; complete T-account borders
</commit_message>
<xml_diff>
--- a/Term_02/BUS 1102-01 Basic Accounting - AY2027-T1/Assignments/Unit2_Assignment.xlsx
+++ b/Term_02/BUS 1102-01 Basic Accounting - AY2027-T1/Assignments/Unit2_Assignment.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="60">
   <si>
     <t>Journal Entries in the Book of Urban Path Co. for the Month of October</t>
   </si>
@@ -183,8 +183,42 @@
     <t>Total</t>
   </si>
   <si>
-    <t>Journal entries are the accounting cycle's starting point: every transaction is first recorded chronologically in a journal, in debit-and-credit form, before it touches any other record (Franklin et al., 2022). Ledgers, organized as T-accounts, then sort each entry into its own account so a business can see a running balance for cash, revenue, or any other item. That organized ledger data is what makes an accurate trial balance possible, since a trial balance simply lists every ledger balance to confirm total debits equal total credits before financial statements get prepared (Franklin et al., 2022).
-Reference: Franklin, M., Graybeal, P., Cooper, D., Bean, L., Burt, I., Carr, S., Collins, D. T., Coram, S., Creech, K., Czyzewski, A., Gauci, M., Greenman, C., Haselkorn, M., Irujo, C., Johnson, C., Khanlarian, C., Lukshaitis, T., Luna, D., Nantz, B, ... Woolley, D. (2022). Principles of accounting, volume 1: Financial accounting. OpenStax. Licensed under CC 4.0. https://openstax.org/details/books/principles-financial-accounting</t>
+    <t>Explanation: Purpose of Journal Entries and Ledgers</t>
+  </si>
+  <si>
+    <t>Journal entries are the accounting cycle's starting point: every transaction is first recorded chronologically in a journal, in debit-and-credit form, before it touches any other record (Franklin et al., 2022). Ledgers, organized as T-accounts, then sort each entry into its own account so a business can see a running balance for cash, revenue, or any other item. That organized ledger data is what makes an accurate trial balance possible, since a trial balance simply lists every ledger balance to confirm total debits equal total credits before financial statements get prepared (Franklin et al., 2022).</t>
+  </si>
+  <si>
+    <t>Reference</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Franklin, M., Graybeal, P., Cooper, D., Bean, L., Burt, I., Carr, S., Collins, D. T., Coram, S., Creech, K., Czyzewski, A., Gauci, M., Greenman, C., Haselkorn, M., Irujo, C., Johnson, C., Khanlarian, C., Lukshaitis, T., Luna, D., Nantz, B., … Woolley, D. (2022). </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Principles of accounting, volume 1: Financial accounting</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>. OpenStax. Licensed under CC 4.0.</t>
+    </r>
+  </si>
+  <si>
+    <t>https://openstax.org/details/books/principles-financial-accounting</t>
   </si>
 </sst>
 </file>
@@ -194,7 +228,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="$#,##0"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -234,6 +268,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -249,7 +291,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -316,6 +358,30 @@
     </border>
     <border>
       <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right/>
       <top/>
       <bottom style="thin">
@@ -332,17 +398,6 @@
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -369,10 +424,10 @@
       <left style="thin">
         <color auto="1"/>
       </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
@@ -382,7 +437,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -391,35 +446,40 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -719,7 +779,7 @@
   <cols>
     <col min="1" max="1" width="3.7109375" customWidth="1"/>
     <col min="2" max="2" width="12.7109375" customWidth="1"/>
-    <col min="3" max="3" width="32.7109375" customWidth="1"/>
+    <col min="3" max="3" width="34.7109375" customWidth="1"/>
     <col min="4" max="4" width="3.7109375" customWidth="1"/>
     <col min="5" max="6" width="14.7109375" customWidth="1"/>
   </cols>
@@ -755,316 +815,407 @@
       <c r="C4" s="6" t="s">
         <v>6</v>
       </c>
+      <c r="D4" s="6"/>
       <c r="E4" s="7">
         <v>50000</v>
       </c>
+      <c r="F4" s="8"/>
     </row>
     <row r="5" spans="2:6">
-      <c r="C5" s="8" t="s">
+      <c r="B5" s="9"/>
+      <c r="C5" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="F5" s="9">
+      <c r="E5" s="9"/>
+      <c r="F5" s="11">
         <v>50000</v>
       </c>
     </row>
     <row r="6" spans="2:6">
-      <c r="C6" s="10" t="s">
+      <c r="B6" s="12"/>
+      <c r="C6" s="13" t="s">
         <v>8</v>
       </c>
+      <c r="D6" s="14"/>
+      <c r="E6" s="12"/>
+      <c r="F6" s="15"/>
     </row>
     <row r="7" spans="2:6">
-      <c r="B7" s="11" t="s">
+      <c r="B7" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="E7" s="12">
+      <c r="E7" s="16">
         <v>10000</v>
       </c>
+      <c r="F7" s="17"/>
     </row>
     <row r="8" spans="2:6">
-      <c r="C8" s="8" t="s">
+      <c r="B8" s="9"/>
+      <c r="C8" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="F8" s="9">
+      <c r="E8" s="9"/>
+      <c r="F8" s="11">
         <v>5000</v>
       </c>
     </row>
     <row r="9" spans="2:6">
-      <c r="C9" s="8" t="s">
+      <c r="B9" s="9"/>
+      <c r="C9" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="F9" s="9">
+      <c r="E9" s="9"/>
+      <c r="F9" s="11">
         <v>5000</v>
       </c>
     </row>
     <row r="10" spans="2:6">
-      <c r="C10" s="13" t="s">
+      <c r="B10" s="5"/>
+      <c r="C10" s="18" t="s">
         <v>13</v>
       </c>
+      <c r="D10" s="6"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="8"/>
     </row>
     <row r="11" spans="2:6">
-      <c r="B11" s="11" t="s">
+      <c r="B11" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="C11" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="E11" s="12">
+      <c r="E11" s="16">
         <v>2000</v>
       </c>
+      <c r="F11" s="17"/>
     </row>
     <row r="12" spans="2:6">
+      <c r="B12" s="12"/>
       <c r="C12" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="F12" s="15">
+      <c r="D12" s="14"/>
+      <c r="E12" s="12"/>
+      <c r="F12" s="19">
         <v>2000</v>
       </c>
     </row>
     <row r="13" spans="2:6">
-      <c r="C13" s="16" t="s">
+      <c r="B13" s="9"/>
+      <c r="C13" s="20" t="s">
         <v>16</v>
       </c>
+      <c r="E13" s="9"/>
+      <c r="F13" s="17"/>
     </row>
     <row r="14" spans="2:6">
-      <c r="B14" s="11" t="s">
+      <c r="B14" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="C14" s="8" t="s">
+      <c r="C14" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="E14" s="12">
+      <c r="E14" s="16">
         <v>1500</v>
       </c>
+      <c r="F14" s="17"/>
     </row>
     <row r="15" spans="2:6">
-      <c r="C15" s="8" t="s">
+      <c r="B15" s="9"/>
+      <c r="C15" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="F15" s="9">
+      <c r="E15" s="9"/>
+      <c r="F15" s="11">
         <v>1500</v>
       </c>
     </row>
     <row r="16" spans="2:6">
-      <c r="C16" s="13" t="s">
+      <c r="B16" s="5"/>
+      <c r="C16" s="18" t="s">
         <v>19</v>
       </c>
+      <c r="D16" s="6"/>
+      <c r="E16" s="5"/>
+      <c r="F16" s="8"/>
     </row>
     <row r="17" spans="2:6">
-      <c r="B17" s="11" t="s">
+      <c r="B17" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="C17" s="8" t="s">
+      <c r="C17" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="E17" s="12">
+      <c r="E17" s="16">
         <v>6000</v>
       </c>
+      <c r="F17" s="17"/>
     </row>
     <row r="18" spans="2:6">
+      <c r="B18" s="12"/>
       <c r="C18" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="F18" s="15">
+      <c r="D18" s="14"/>
+      <c r="E18" s="12"/>
+      <c r="F18" s="19">
         <v>6000</v>
       </c>
     </row>
     <row r="19" spans="2:6">
-      <c r="C19" s="16" t="s">
+      <c r="B19" s="9"/>
+      <c r="C19" s="20" t="s">
         <v>23</v>
       </c>
+      <c r="E19" s="9"/>
+      <c r="F19" s="17"/>
     </row>
     <row r="20" spans="2:6">
-      <c r="B20" s="11" t="s">
+      <c r="B20" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="C20" s="8" t="s">
+      <c r="C20" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="E20" s="12">
+      <c r="E20" s="16">
         <v>1000</v>
       </c>
+      <c r="F20" s="17"/>
     </row>
     <row r="21" spans="2:6">
-      <c r="C21" s="8" t="s">
+      <c r="B21" s="9"/>
+      <c r="C21" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="F21" s="9">
+      <c r="E21" s="9"/>
+      <c r="F21" s="11">
         <v>1000</v>
       </c>
     </row>
     <row r="22" spans="2:6">
-      <c r="C22" s="13" t="s">
+      <c r="B22" s="5"/>
+      <c r="C22" s="18" t="s">
         <v>26</v>
       </c>
+      <c r="D22" s="6"/>
+      <c r="E22" s="5"/>
+      <c r="F22" s="8"/>
     </row>
     <row r="23" spans="2:6">
-      <c r="B23" s="11" t="s">
+      <c r="B23" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="C23" s="8" t="s">
+      <c r="C23" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="E23" s="12">
+      <c r="E23" s="16">
         <v>4000</v>
       </c>
+      <c r="F23" s="17"/>
     </row>
     <row r="24" spans="2:6">
+      <c r="B24" s="12"/>
       <c r="C24" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="F24" s="15">
+      <c r="D24" s="14"/>
+      <c r="E24" s="12"/>
+      <c r="F24" s="19">
         <v>4000</v>
       </c>
     </row>
     <row r="25" spans="2:6">
-      <c r="C25" s="16" t="s">
+      <c r="B25" s="9"/>
+      <c r="C25" s="20" t="s">
         <v>29</v>
       </c>
+      <c r="E25" s="9"/>
+      <c r="F25" s="17"/>
     </row>
     <row r="26" spans="2:6">
-      <c r="B26" s="11" t="s">
+      <c r="B26" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="C26" s="8" t="s">
+      <c r="C26" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="E26" s="12">
+      <c r="E26" s="16">
         <v>3500</v>
       </c>
+      <c r="F26" s="17"/>
     </row>
     <row r="27" spans="2:6">
-      <c r="C27" s="8" t="s">
+      <c r="B27" s="9"/>
+      <c r="C27" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="F27" s="9">
+      <c r="E27" s="9"/>
+      <c r="F27" s="11">
         <v>3500</v>
       </c>
     </row>
     <row r="28" spans="2:6">
-      <c r="C28" s="13" t="s">
+      <c r="B28" s="5"/>
+      <c r="C28" s="18" t="s">
         <v>32</v>
       </c>
+      <c r="D28" s="6"/>
+      <c r="E28" s="5"/>
+      <c r="F28" s="8"/>
     </row>
     <row r="29" spans="2:6">
-      <c r="B29" s="11" t="s">
+      <c r="B29" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="C29" s="8" t="s">
+      <c r="C29" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="E29" s="12">
+      <c r="E29" s="16">
         <v>2000</v>
       </c>
+      <c r="F29" s="17"/>
     </row>
     <row r="30" spans="2:6">
+      <c r="B30" s="12"/>
       <c r="C30" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="F30" s="15">
+      <c r="D30" s="14"/>
+      <c r="E30" s="12"/>
+      <c r="F30" s="19">
         <v>2000</v>
       </c>
     </row>
     <row r="31" spans="2:6">
-      <c r="C31" s="16" t="s">
+      <c r="B31" s="9"/>
+      <c r="C31" s="20" t="s">
         <v>35</v>
       </c>
+      <c r="E31" s="9"/>
+      <c r="F31" s="17"/>
     </row>
     <row r="32" spans="2:6">
-      <c r="B32" s="11" t="s">
+      <c r="B32" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="C32" s="8" t="s">
+      <c r="C32" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="E32" s="12">
+      <c r="E32" s="16">
         <v>1200</v>
       </c>
+      <c r="F32" s="17"/>
     </row>
     <row r="33" spans="2:6">
-      <c r="C33" s="8" t="s">
+      <c r="B33" s="9"/>
+      <c r="C33" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="F33" s="9">
+      <c r="E33" s="9"/>
+      <c r="F33" s="11">
         <v>1200</v>
       </c>
     </row>
     <row r="34" spans="2:6">
-      <c r="C34" s="13" t="s">
+      <c r="B34" s="5"/>
+      <c r="C34" s="18" t="s">
         <v>38</v>
       </c>
+      <c r="D34" s="6"/>
+      <c r="E34" s="5"/>
+      <c r="F34" s="8"/>
     </row>
     <row r="35" spans="2:6">
-      <c r="B35" s="11" t="s">
+      <c r="B35" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="C35" s="8" t="s">
+      <c r="C35" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="E35" s="12">
+      <c r="E35" s="16">
         <v>7500</v>
       </c>
+      <c r="F35" s="17"/>
     </row>
     <row r="36" spans="2:6">
+      <c r="B36" s="12"/>
       <c r="C36" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="F36" s="15">
+      <c r="D36" s="14"/>
+      <c r="E36" s="12"/>
+      <c r="F36" s="19">
         <v>7500</v>
       </c>
     </row>
     <row r="37" spans="2:6">
-      <c r="C37" s="16" t="s">
+      <c r="B37" s="9"/>
+      <c r="C37" s="20" t="s">
         <v>40</v>
       </c>
+      <c r="E37" s="9"/>
+      <c r="F37" s="17"/>
     </row>
     <row r="38" spans="2:6">
-      <c r="B38" s="11" t="s">
+      <c r="B38" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="C38" s="8" t="s">
+      <c r="C38" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="E38" s="12">
+      <c r="E38" s="16">
         <v>1000</v>
       </c>
+      <c r="F38" s="17"/>
     </row>
     <row r="39" spans="2:6">
-      <c r="C39" s="8" t="s">
+      <c r="B39" s="9"/>
+      <c r="C39" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="F39" s="9">
+      <c r="E39" s="9"/>
+      <c r="F39" s="11">
         <v>1000</v>
       </c>
     </row>
     <row r="40" spans="2:6">
-      <c r="C40" s="13" t="s">
+      <c r="B40" s="5"/>
+      <c r="C40" s="18" t="s">
         <v>42</v>
       </c>
+      <c r="D40" s="6"/>
+      <c r="E40" s="5"/>
+      <c r="F40" s="8"/>
     </row>
     <row r="41" spans="2:6">
-      <c r="B41" s="11" t="s">
+      <c r="B41" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="C41" s="8" t="s">
+      <c r="C41" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="E41" s="12">
+      <c r="E41" s="16">
         <v>3000</v>
       </c>
+      <c r="F41" s="17"/>
     </row>
     <row r="42" spans="2:6">
+      <c r="B42" s="12"/>
       <c r="C42" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="F42" s="15">
+      <c r="D42" s="14"/>
+      <c r="E42" s="12"/>
+      <c r="F42" s="19">
         <v>3000</v>
       </c>
     </row>
     <row r="43" spans="2:6">
-      <c r="C43" s="16" t="s">
+      <c r="C43" s="20" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1094,404 +1245,514 @@
     <col min="14" max="14" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="3:14">
-      <c r="C1" s="17" t="s">
+    <row r="1" spans="2:14">
+      <c r="B1" s="14"/>
+      <c r="C1" s="21" t="s">
         <v>45</v>
       </c>
-      <c r="K1" s="18" t="s">
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="K1" s="22" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="2" spans="3:14">
-      <c r="C2" s="19" t="s">
+    <row r="2" spans="2:14">
+      <c r="B2" s="14"/>
+      <c r="C2" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="20" t="s">
+      <c r="D2" s="14"/>
+      <c r="E2" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="K2" s="19" t="s">
+      <c r="J2" s="14"/>
+      <c r="K2" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="M2" s="20" t="s">
+      <c r="L2" s="14"/>
+      <c r="M2" s="24" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="3:14">
-      <c r="C3" s="21" t="s">
+    <row r="3" spans="2:14">
+      <c r="C3" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="22">
+      <c r="D3" s="25">
         <v>50000</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="F3" s="22">
+      <c r="F3" s="25">
         <v>5000</v>
       </c>
-      <c r="K3" s="23" t="s">
+      <c r="K3" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="L3" s="22">
+      <c r="L3" s="25">
         <v>1500</v>
       </c>
     </row>
-    <row r="4" spans="3:14">
-      <c r="C4" s="23" t="s">
+    <row r="4" spans="2:14">
+      <c r="C4" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="D4" s="22">
+      <c r="D4" s="25">
         <v>4000</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="E4" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F4" s="22">
+      <c r="F4" s="25">
         <v>2000</v>
       </c>
-      <c r="K4" s="24" t="s">
+      <c r="K4" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="L4" s="25">
+      <c r="L4" s="27">
         <v>1500</v>
       </c>
     </row>
-    <row r="5" spans="3:14">
-      <c r="C5" s="23" t="s">
+    <row r="5" spans="2:14">
+      <c r="C5" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="D5" s="22">
+      <c r="D5" s="25">
         <v>7500</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="E5" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="F5" s="22">
+      <c r="F5" s="25">
         <v>1000</v>
       </c>
-    </row>
-    <row r="6" spans="3:14">
-      <c r="E6" s="8" t="s">
+      <c r="K5" s="17"/>
+    </row>
+    <row r="6" spans="2:14">
+      <c r="C6" s="17"/>
+      <c r="E6" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="F6" s="22">
+      <c r="F6" s="25">
         <v>3500</v>
       </c>
     </row>
-    <row r="7" spans="3:14">
-      <c r="E7" s="8" t="s">
+    <row r="7" spans="2:14">
+      <c r="C7" s="17"/>
+      <c r="E7" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="F7" s="22">
+      <c r="F7" s="25">
         <v>2000</v>
       </c>
     </row>
-    <row r="8" spans="3:14">
-      <c r="E8" s="8" t="s">
+    <row r="8" spans="2:14">
+      <c r="C8" s="17"/>
+      <c r="E8" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="F8" s="22">
+      <c r="F8" s="25">
         <v>3000</v>
       </c>
-      <c r="K8" s="18" t="s">
+      <c r="K8" s="22" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="3:14">
-      <c r="C9" s="24" t="s">
+    <row r="9" spans="2:14">
+      <c r="C9" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="D9" s="25">
+      <c r="D9" s="27">
         <v>45000</v>
       </c>
-      <c r="K9" s="19" t="s">
+      <c r="J9" s="14"/>
+      <c r="K9" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="M9" s="20" t="s">
+      <c r="L9" s="14"/>
+      <c r="M9" s="24" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="3:14">
-      <c r="K10" s="23" t="s">
+    <row r="10" spans="2:14">
+      <c r="C10" s="17"/>
+      <c r="K10" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="L10" s="22">
+      <c r="L10" s="25">
         <v>6000</v>
       </c>
-      <c r="M10" s="8" t="s">
+      <c r="M10" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="N10" s="22">
+      <c r="N10" s="25">
         <v>4000</v>
       </c>
     </row>
-    <row r="11" spans="3:14">
-      <c r="K11" s="24" t="s">
+    <row r="11" spans="2:14">
+      <c r="C11" s="17"/>
+      <c r="K11" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="L11" s="25">
+      <c r="L11" s="27">
         <v>2000</v>
       </c>
     </row>
-    <row r="17" spans="3:14">
-      <c r="C17" s="18" t="s">
+    <row r="12" spans="2:14">
+      <c r="C12" s="17"/>
+      <c r="K12" s="17"/>
+    </row>
+    <row r="17" spans="2:14">
+      <c r="C17" s="22" t="s">
         <v>48</v>
       </c>
-      <c r="K17" s="18" t="s">
+      <c r="K17" s="22" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="18" spans="3:14">
-      <c r="C18" s="19" t="s">
+    <row r="18" spans="2:14">
+      <c r="B18" s="14"/>
+      <c r="C18" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="E18" s="20" t="s">
+      <c r="D18" s="14"/>
+      <c r="E18" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="K18" s="19" t="s">
+      <c r="J18" s="14"/>
+      <c r="K18" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="M18" s="20" t="s">
+      <c r="L18" s="14"/>
+      <c r="M18" s="24" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="19" spans="3:14">
-      <c r="E19" s="8" t="s">
+    <row r="19" spans="2:14">
+      <c r="C19" s="8"/>
+      <c r="E19" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="F19" s="22">
+      <c r="F19" s="25">
         <v>50000</v>
       </c>
-      <c r="M19" s="8" t="s">
+      <c r="K19" s="17"/>
+      <c r="M19" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="N19" s="22">
+      <c r="N19" s="25">
         <v>6000</v>
       </c>
     </row>
-    <row r="20" spans="3:14">
-      <c r="E20" s="26" t="s">
+    <row r="20" spans="2:14">
+      <c r="C20" s="17"/>
+      <c r="E20" s="28" t="s">
         <v>46</v>
       </c>
-      <c r="F20" s="25">
+      <c r="F20" s="27">
         <v>50000</v>
       </c>
-      <c r="M20" s="8" t="s">
+      <c r="K20" s="17"/>
+      <c r="M20" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="N20" s="22">
+      <c r="N20" s="25">
         <v>7500</v>
       </c>
     </row>
-    <row r="21" spans="3:14">
-      <c r="M21" s="26" t="s">
+    <row r="21" spans="2:14">
+      <c r="K21" s="17"/>
+      <c r="M21" s="28" t="s">
         <v>46</v>
       </c>
-      <c r="N21" s="25">
+      <c r="N21" s="27">
         <v>13500</v>
       </c>
     </row>
-    <row r="26" spans="3:14">
-      <c r="C26" s="18" t="s">
+    <row r="26" spans="2:14">
+      <c r="C26" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="K26" s="18" t="s">
+      <c r="K26" s="22" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="27" spans="3:14">
-      <c r="C27" s="19" t="s">
+    <row r="27" spans="2:14">
+      <c r="B27" s="14"/>
+      <c r="C27" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="E27" s="20" t="s">
+      <c r="D27" s="14"/>
+      <c r="E27" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="K27" s="19" t="s">
+      <c r="J27" s="14"/>
+      <c r="K27" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="M27" s="20" t="s">
+      <c r="L27" s="14"/>
+      <c r="M27" s="24" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="28" spans="3:14">
-      <c r="C28" s="23" t="s">
+    <row r="28" spans="2:14">
+      <c r="C28" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="D28" s="22">
+      <c r="D28" s="25">
         <v>10000</v>
       </c>
-      <c r="K28" s="23" t="s">
+      <c r="K28" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="L28" s="22">
+      <c r="L28" s="25">
         <v>3500</v>
       </c>
     </row>
-    <row r="29" spans="3:14">
-      <c r="C29" s="23" t="s">
+    <row r="29" spans="2:14">
+      <c r="C29" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="D29" s="22">
+      <c r="D29" s="25">
         <v>1000</v>
       </c>
-      <c r="K29" s="24" t="s">
+      <c r="K29" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="L29" s="25">
+      <c r="L29" s="27">
         <v>3500</v>
       </c>
     </row>
+    <row r="30" spans="2:14">
+      <c r="C30" s="17"/>
+      <c r="K30" s="17"/>
+    </row>
+    <row r="31" spans="2:14">
+      <c r="C31" s="17"/>
+    </row>
     <row r="33" spans="2:13">
-      <c r="B33" s="26" t="s">
+      <c r="B33" s="28" t="s">
         <v>46</v>
       </c>
-      <c r="C33" s="25">
+      <c r="C33" s="27">
         <v>11000</v>
       </c>
     </row>
     <row r="35" spans="2:13">
-      <c r="C35" s="18" t="s">
+      <c r="C35" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="K35" s="18" t="s">
+      <c r="K35" s="22" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="36" spans="2:13">
-      <c r="C36" s="19" t="s">
+      <c r="B36" s="14"/>
+      <c r="C36" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="E36" s="20" t="s">
+      <c r="D36" s="14"/>
+      <c r="E36" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="K36" s="19" t="s">
+      <c r="J36" s="14"/>
+      <c r="K36" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="M36" s="20" t="s">
+      <c r="L36" s="14"/>
+      <c r="M36" s="24" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="37" spans="2:13">
-      <c r="C37" s="8" t="s">
+      <c r="C37" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="D37" s="27">
+      <c r="D37" s="29">
         <v>1000</v>
       </c>
-      <c r="E37" s="8" t="s">
+      <c r="E37" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="F37" s="22">
+      <c r="F37" s="25">
         <v>5000</v>
       </c>
-      <c r="K37" s="23" t="s">
+      <c r="K37" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="L37" s="22">
+      <c r="L37" s="25">
         <v>1200</v>
       </c>
     </row>
     <row r="38" spans="2:13">
-      <c r="C38" s="8" t="s">
+      <c r="C38" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="D38" s="27">
+      <c r="D38" s="29">
         <v>3000</v>
       </c>
-      <c r="E38" s="8" t="s">
+      <c r="E38" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="F38" s="22">
+      <c r="F38" s="25">
         <v>1500</v>
       </c>
-      <c r="K38" s="24" t="s">
+      <c r="K38" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="L38" s="25">
+      <c r="L38" s="27">
         <v>1200</v>
       </c>
     </row>
     <row r="39" spans="2:13">
-      <c r="E39" s="8" t="s">
+      <c r="C39" s="17"/>
+      <c r="E39" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="F39" s="22">
+      <c r="F39" s="25">
         <v>1200</v>
       </c>
+      <c r="K39" s="17"/>
     </row>
     <row r="40" spans="2:13">
-      <c r="E40" s="8" t="s">
+      <c r="D40" s="30"/>
+      <c r="E40" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="F40" s="22">
+      <c r="F40" s="25">
         <v>1000</v>
       </c>
     </row>
     <row r="41" spans="2:13">
-      <c r="E41" s="26" t="s">
+      <c r="E41" s="28" t="s">
         <v>46</v>
       </c>
-      <c r="F41" s="25">
+      <c r="F41" s="27">
         <v>4700</v>
       </c>
     </row>
     <row r="44" spans="2:13">
-      <c r="C44" s="18" t="s">
+      <c r="C44" s="22" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="45" spans="2:13">
-      <c r="C45" s="19" t="s">
+      <c r="B45" s="14"/>
+      <c r="C45" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="E45" s="20" t="s">
+      <c r="D45" s="14"/>
+      <c r="E45" s="24" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="46" spans="2:13">
-      <c r="C46" s="8" t="s">
+      <c r="C46" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="D46" s="27">
+      <c r="D46" s="29">
         <v>2000</v>
       </c>
     </row>
     <row r="47" spans="2:13">
-      <c r="C47" s="24" t="s">
+      <c r="C47" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="D47" s="25">
+      <c r="D47" s="27">
         <v>2000</v>
       </c>
     </row>
-    <row r="75" spans="3:5">
-      <c r="C75" s="18" t="s">
+    <row r="53" spans="2:13">
+      <c r="B53" s="14"/>
+      <c r="C53" s="15"/>
+      <c r="D53" s="14"/>
+      <c r="E53" s="14"/>
+      <c r="J53" s="14"/>
+      <c r="K53" s="15"/>
+      <c r="L53" s="14"/>
+      <c r="M53" s="14"/>
+    </row>
+    <row r="54" spans="2:13">
+      <c r="C54" s="17"/>
+      <c r="K54" s="8"/>
+    </row>
+    <row r="55" spans="2:13">
+      <c r="C55" s="17"/>
+      <c r="K55" s="17"/>
+    </row>
+    <row r="62" spans="2:13">
+      <c r="B62" s="14"/>
+      <c r="C62" s="15"/>
+      <c r="D62" s="14"/>
+      <c r="E62" s="14"/>
+      <c r="J62" s="14"/>
+      <c r="K62" s="15"/>
+      <c r="L62" s="14"/>
+      <c r="M62" s="14"/>
+    </row>
+    <row r="63" spans="2:13">
+      <c r="C63" s="17"/>
+      <c r="K63" s="8"/>
+    </row>
+    <row r="64" spans="2:13">
+      <c r="C64" s="17"/>
+      <c r="K64" s="17"/>
+    </row>
+    <row r="68" spans="2:13">
+      <c r="B68" s="14"/>
+      <c r="C68" s="15"/>
+      <c r="D68" s="14"/>
+      <c r="E68" s="14"/>
+      <c r="J68" s="14"/>
+      <c r="K68" s="15"/>
+      <c r="L68" s="14"/>
+      <c r="M68" s="14"/>
+    </row>
+    <row r="69" spans="2:13">
+      <c r="C69" s="17"/>
+      <c r="K69" s="8"/>
+    </row>
+    <row r="70" spans="2:13">
+      <c r="C70" s="17"/>
+      <c r="K70" s="17"/>
+    </row>
+    <row r="75" spans="2:13">
+      <c r="C75" s="22" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="76" spans="3:5">
-      <c r="C76" s="19" t="s">
+    <row r="76" spans="2:13">
+      <c r="B76" s="14"/>
+      <c r="C76" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="E76" s="20" t="s">
+      <c r="D76" s="14"/>
+      <c r="E76" s="24" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="77" spans="3:5">
-      <c r="C77" s="21" t="s">
+      <c r="J76" s="14"/>
+      <c r="K76" s="15"/>
+      <c r="L76" s="14"/>
+      <c r="M76" s="14"/>
+    </row>
+    <row r="77" spans="2:13">
+      <c r="C77" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="D77" s="22">
+      <c r="D77" s="25">
         <v>2000</v>
       </c>
-    </row>
-    <row r="78" spans="3:5">
-      <c r="C78" s="24" t="s">
+      <c r="K77" s="8"/>
+    </row>
+    <row r="78" spans="2:13">
+      <c r="C78" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="D78" s="25">
+      <c r="D78" s="27">
         <v>2000</v>
       </c>
+      <c r="K78" s="17"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1500,10 +1761,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N22"/>
+  <dimension ref="A1:N25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="28.7109375" customWidth="1"/>
+    <col min="1" max="1" width="30.7109375" customWidth="1"/>
     <col min="2" max="3" width="15.7109375" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1515,13 +1776,13 @@
       <c r="C1" s="1"/>
     </row>
     <row r="2" spans="1:3">
-      <c r="A2" s="28" t="s">
+      <c r="A2" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="28" t="s">
+      <c r="B2" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="29" t="s">
+      <c r="C2" s="32" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1529,39 +1790,44 @@
       <c r="A3" s="30" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="27">
+      <c r="B3" s="29">
         <v>45000</v>
       </c>
+      <c r="C3" s="9"/>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="30" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="27">
+      <c r="B4" s="29">
         <v>2000</v>
       </c>
+      <c r="C4" s="9"/>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="27">
+      <c r="B5" s="29">
         <v>1500</v>
       </c>
+      <c r="C5" s="9"/>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="27">
+      <c r="B6" s="29">
         <v>11000</v>
       </c>
+      <c r="C6" s="9"/>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="12">
+      <c r="B7" s="30"/>
+      <c r="C7" s="16">
         <v>4700</v>
       </c>
     </row>
@@ -1569,7 +1835,8 @@
       <c r="A8" s="30" t="s">
         <v>53</v>
       </c>
-      <c r="C8" s="12">
+      <c r="B8" s="30"/>
+      <c r="C8" s="16">
         <v>50000</v>
       </c>
     </row>
@@ -1577,15 +1844,17 @@
       <c r="A9" s="30" t="s">
         <v>34</v>
       </c>
-      <c r="B9" s="27">
+      <c r="B9" s="29">
         <v>2000</v>
       </c>
+      <c r="C9" s="9"/>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" s="30" t="s">
         <v>49</v>
       </c>
-      <c r="C10" s="12">
+      <c r="B10" s="30"/>
+      <c r="C10" s="16">
         <v>13500</v>
       </c>
     </row>
@@ -1593,140 +1862,203 @@
       <c r="A11" s="30" t="s">
         <v>31</v>
       </c>
-      <c r="B11" s="27">
+      <c r="B11" s="29">
         <v>3500</v>
       </c>
+      <c r="C11" s="9"/>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="27">
+      <c r="B12" s="29">
         <v>2000</v>
       </c>
+      <c r="C12" s="9"/>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" s="30" t="s">
         <v>37</v>
       </c>
-      <c r="B13" s="27">
+      <c r="B13" s="29">
         <v>1200</v>
       </c>
+      <c r="C13" s="9"/>
     </row>
     <row r="14" spans="1:3">
-      <c r="A14" s="31" t="s">
+      <c r="A14" s="33" t="s">
         <v>54</v>
       </c>
-      <c r="B14" s="32">
+      <c r="B14" s="34">
         <v>68200</v>
       </c>
-      <c r="C14" s="33">
+      <c r="C14" s="35">
         <v>68200</v>
       </c>
     </row>
-    <row r="17" spans="1:14" ht="30" customHeight="1">
-      <c r="A17" s="34" t="s">
+    <row r="15" spans="1:3">
+      <c r="A15" s="30"/>
+      <c r="B15" s="30"/>
+      <c r="C15" s="9"/>
+    </row>
+    <row r="16" spans="1:3">
+      <c r="A16" s="28" t="s">
         <v>55</v>
       </c>
-      <c r="B17" s="34"/>
-      <c r="C17" s="34"/>
-      <c r="D17" s="34"/>
-      <c r="E17" s="34"/>
-      <c r="F17" s="34"/>
-      <c r="G17" s="34"/>
-      <c r="H17" s="34"/>
-      <c r="I17" s="34"/>
-      <c r="J17" s="34"/>
-      <c r="K17" s="34"/>
-      <c r="L17" s="34"/>
-      <c r="M17" s="34"/>
-      <c r="N17" s="34"/>
+      <c r="B16" s="30"/>
+      <c r="C16" s="9"/>
+    </row>
+    <row r="17" spans="1:14">
+      <c r="A17" s="36" t="s">
+        <v>56</v>
+      </c>
+      <c r="B17" s="36"/>
+      <c r="C17" s="36"/>
+      <c r="D17" s="36"/>
+      <c r="E17" s="36"/>
+      <c r="F17" s="36"/>
+      <c r="G17" s="36"/>
+      <c r="H17" s="36"/>
+      <c r="I17" s="36"/>
+      <c r="J17" s="36"/>
+      <c r="K17" s="36"/>
+      <c r="L17" s="36"/>
+      <c r="M17" s="36"/>
+      <c r="N17" s="36"/>
     </row>
     <row r="18" spans="1:14">
-      <c r="A18" s="34"/>
-      <c r="B18" s="34"/>
-      <c r="C18" s="34"/>
-      <c r="D18" s="34"/>
-      <c r="E18" s="34"/>
-      <c r="F18" s="34"/>
-      <c r="G18" s="34"/>
-      <c r="H18" s="34"/>
-      <c r="I18" s="34"/>
-      <c r="J18" s="34"/>
-      <c r="K18" s="34"/>
-      <c r="L18" s="34"/>
-      <c r="M18" s="34"/>
-      <c r="N18" s="34"/>
+      <c r="A18" s="36"/>
+      <c r="B18" s="36"/>
+      <c r="C18" s="36"/>
+      <c r="D18" s="36"/>
+      <c r="E18" s="36"/>
+      <c r="F18" s="36"/>
+      <c r="G18" s="36"/>
+      <c r="H18" s="36"/>
+      <c r="I18" s="36"/>
+      <c r="J18" s="36"/>
+      <c r="K18" s="36"/>
+      <c r="L18" s="36"/>
+      <c r="M18" s="36"/>
+      <c r="N18" s="36"/>
     </row>
     <row r="19" spans="1:14">
-      <c r="A19" s="34"/>
-      <c r="B19" s="34"/>
-      <c r="C19" s="34"/>
-      <c r="D19" s="34"/>
-      <c r="E19" s="34"/>
-      <c r="F19" s="34"/>
-      <c r="G19" s="34"/>
-      <c r="H19" s="34"/>
-      <c r="I19" s="34"/>
-      <c r="J19" s="34"/>
-      <c r="K19" s="34"/>
-      <c r="L19" s="34"/>
-      <c r="M19" s="34"/>
-      <c r="N19" s="34"/>
+      <c r="A19" s="36"/>
+      <c r="B19" s="36"/>
+      <c r="C19" s="36"/>
+      <c r="D19" s="36"/>
+      <c r="E19" s="36"/>
+      <c r="F19" s="36"/>
+      <c r="G19" s="36"/>
+      <c r="H19" s="36"/>
+      <c r="I19" s="36"/>
+      <c r="J19" s="36"/>
+      <c r="K19" s="36"/>
+      <c r="L19" s="36"/>
+      <c r="M19" s="36"/>
+      <c r="N19" s="36"/>
     </row>
     <row r="20" spans="1:14">
-      <c r="A20" s="34"/>
-      <c r="B20" s="34"/>
-      <c r="C20" s="34"/>
-      <c r="D20" s="34"/>
-      <c r="E20" s="34"/>
-      <c r="F20" s="34"/>
-      <c r="G20" s="34"/>
-      <c r="H20" s="34"/>
-      <c r="I20" s="34"/>
-      <c r="J20" s="34"/>
-      <c r="K20" s="34"/>
-      <c r="L20" s="34"/>
-      <c r="M20" s="34"/>
-      <c r="N20" s="34"/>
+      <c r="A20" s="36"/>
+      <c r="B20" s="36"/>
+      <c r="C20" s="36"/>
+      <c r="D20" s="36"/>
+      <c r="E20" s="36"/>
+      <c r="F20" s="36"/>
+      <c r="G20" s="36"/>
+      <c r="H20" s="36"/>
+      <c r="I20" s="36"/>
+      <c r="J20" s="36"/>
+      <c r="K20" s="36"/>
+      <c r="L20" s="36"/>
+      <c r="M20" s="36"/>
+      <c r="N20" s="36"/>
     </row>
     <row r="21" spans="1:14">
-      <c r="A21" s="34"/>
-      <c r="B21" s="34"/>
-      <c r="C21" s="34"/>
-      <c r="D21" s="34"/>
-      <c r="E21" s="34"/>
-      <c r="F21" s="34"/>
-      <c r="G21" s="34"/>
-      <c r="H21" s="34"/>
-      <c r="I21" s="34"/>
-      <c r="J21" s="34"/>
-      <c r="K21" s="34"/>
-      <c r="L21" s="34"/>
-      <c r="M21" s="34"/>
-      <c r="N21" s="34"/>
+      <c r="A21" s="36"/>
+      <c r="B21" s="36"/>
+      <c r="C21" s="36"/>
+      <c r="D21" s="36"/>
+      <c r="E21" s="36"/>
+      <c r="F21" s="36"/>
+      <c r="G21" s="36"/>
+      <c r="H21" s="36"/>
+      <c r="I21" s="36"/>
+      <c r="J21" s="36"/>
+      <c r="K21" s="36"/>
+      <c r="L21" s="36"/>
+      <c r="M21" s="36"/>
+      <c r="N21" s="36"/>
     </row>
     <row r="22" spans="1:14">
-      <c r="A22" s="34"/>
-      <c r="B22" s="34"/>
-      <c r="C22" s="34"/>
-      <c r="D22" s="34"/>
-      <c r="E22" s="34"/>
-      <c r="F22" s="34"/>
-      <c r="G22" s="34"/>
-      <c r="H22" s="34"/>
-      <c r="I22" s="34"/>
-      <c r="J22" s="34"/>
-      <c r="K22" s="34"/>
-      <c r="L22" s="34"/>
-      <c r="M22" s="34"/>
-      <c r="N22" s="34"/>
+      <c r="A22" s="28" t="s">
+        <v>57</v>
+      </c>
+      <c r="B22" s="37"/>
+      <c r="C22" s="38"/>
+    </row>
+    <row r="23" spans="1:14">
+      <c r="A23" s="36" t="s">
+        <v>58</v>
+      </c>
+      <c r="B23" s="36"/>
+      <c r="C23" s="36"/>
+      <c r="D23" s="36"/>
+      <c r="E23" s="36"/>
+      <c r="F23" s="36"/>
+      <c r="G23" s="36"/>
+      <c r="H23" s="36"/>
+      <c r="I23" s="36"/>
+      <c r="J23" s="36"/>
+      <c r="K23" s="36"/>
+      <c r="L23" s="36"/>
+      <c r="M23" s="36"/>
+      <c r="N23" s="36"/>
+    </row>
+    <row r="24" spans="1:14">
+      <c r="A24" s="36"/>
+      <c r="B24" s="36"/>
+      <c r="C24" s="36"/>
+      <c r="D24" s="36"/>
+      <c r="E24" s="36"/>
+      <c r="F24" s="36"/>
+      <c r="G24" s="36"/>
+      <c r="H24" s="36"/>
+      <c r="I24" s="36"/>
+      <c r="J24" s="36"/>
+      <c r="K24" s="36"/>
+      <c r="L24" s="36"/>
+      <c r="M24" s="36"/>
+      <c r="N24" s="36"/>
+    </row>
+    <row r="25" spans="1:14">
+      <c r="A25" s="39" t="s">
+        <v>59</v>
+      </c>
+      <c r="B25" s="36"/>
+      <c r="C25" s="36"/>
+      <c r="D25" s="36"/>
+      <c r="E25" s="36"/>
+      <c r="F25" s="36"/>
+      <c r="G25" s="36"/>
+      <c r="H25" s="36"/>
+      <c r="I25" s="36"/>
+      <c r="J25" s="36"/>
+      <c r="K25" s="36"/>
+      <c r="L25" s="36"/>
+      <c r="M25" s="36"/>
+      <c r="N25" s="36"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="4">
     <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A17:N22"/>
+    <mergeCell ref="A17:N21"/>
+    <mergeCell ref="A23:N24"/>
+    <mergeCell ref="A25:N25"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="A25" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix T-account column alignment to template layout (dates in B/J, amounts in C/K) and restore template column widths
</commit_message>
<xml_diff>
--- a/Term_02/BUS 1102-01 Basic Accounting - AY2027-T1/Assignments/Unit2_Assignment.xlsx
+++ b/Term_02/BUS 1102-01 Basic Accounting - AY2027-T1/Assignments/Unit2_Assignment.xlsx
@@ -159,19 +159,19 @@
     <t>Balance</t>
   </si>
   <si>
+    <t>Common Stock account</t>
+  </si>
+  <si>
+    <t>Rent account</t>
+  </si>
+  <si>
+    <t>Dividend account</t>
+  </si>
+  <si>
     <t>Office Supply</t>
   </si>
   <si>
-    <t>Common Stock account</t>
-  </si>
-  <si>
     <t>Service Revenue</t>
-  </si>
-  <si>
-    <t>Rent account</t>
-  </si>
-  <si>
-    <t>Dividend account</t>
   </si>
   <si>
     <t>Trial Balance Urban Path Co.</t>
@@ -291,7 +291,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -420,24 +420,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -463,22 +450,21 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -777,11 +763,13 @@
   <dimension ref="B2:F43"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="3.7109375" customWidth="1"/>
-    <col min="2" max="2" width="12.7109375" customWidth="1"/>
-    <col min="3" max="3" width="34.7109375" customWidth="1"/>
-    <col min="4" max="4" width="3.7109375" customWidth="1"/>
-    <col min="5" max="6" width="14.7109375" customWidth="1"/>
+    <col min="1" max="1" width="9.85546875" customWidth="1"/>
+    <col min="2" max="2" width="13.42578125" customWidth="1"/>
+    <col min="3" max="3" width="45.5703125" customWidth="1"/>
+    <col min="4" max="4" width="6.140625" customWidth="1"/>
+    <col min="5" max="5" width="13.7109375" customWidth="1"/>
+    <col min="6" max="6" width="18.85546875" customWidth="1"/>
+    <col min="7" max="7" width="9.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:6">
@@ -1229,23 +1217,20 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="B1:N78"/>
+  <dimension ref="B1:M78"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="2.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="10.7109375" customWidth="1"/>
-    <col min="4" max="4" width="12.7109375" customWidth="1"/>
-    <col min="5" max="5" width="10.7109375" customWidth="1"/>
-    <col min="6" max="6" width="12.7109375" customWidth="1"/>
-    <col min="10" max="10" width="2.7109375" customWidth="1"/>
-    <col min="11" max="11" width="10.7109375" customWidth="1"/>
-    <col min="12" max="12" width="12.7109375" customWidth="1"/>
-    <col min="13" max="13" width="10.7109375" customWidth="1"/>
-    <col min="14" max="14" width="12.7109375" customWidth="1"/>
+    <col min="2" max="2" width="19.140625" customWidth="1"/>
+    <col min="3" max="3" width="8.5703125" customWidth="1"/>
+    <col min="4" max="4" width="17.140625" customWidth="1"/>
+    <col min="5" max="5" width="8.5703125" customWidth="1"/>
+    <col min="10" max="10" width="16.140625" customWidth="1"/>
+    <col min="11" max="11" width="10.140625" customWidth="1"/>
+    <col min="12" max="12" width="17.140625" customWidth="1"/>
+    <col min="13" max="13" width="11.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:14">
+    <row r="1" spans="2:13">
       <c r="B1" s="14"/>
       <c r="C1" s="21" t="s">
         <v>45</v>
@@ -1253,10 +1238,10 @@
       <c r="D1" s="14"/>
       <c r="E1" s="14"/>
       <c r="K1" s="22" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="2" spans="2:14">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="2" spans="2:13">
       <c r="B2" s="14"/>
       <c r="C2" s="23" t="s">
         <v>3</v>
@@ -1274,96 +1259,96 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="2:14">
-      <c r="C3" s="8" t="s">
+    <row r="3" spans="2:13">
+      <c r="B3" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="25">
+      <c r="C3" s="25">
         <v>50000</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="D3" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="F3" s="25">
+      <c r="E3" s="26">
         <v>5000</v>
       </c>
-      <c r="K3" s="17" t="s">
+      <c r="J3" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="L3" s="25">
+      <c r="K3" s="11">
         <v>1500</v>
       </c>
     </row>
-    <row r="4" spans="2:14">
-      <c r="C4" s="17" t="s">
+    <row r="4" spans="2:13">
+      <c r="B4" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="D4" s="25">
+      <c r="C4" s="11">
         <v>4000</v>
       </c>
-      <c r="E4" s="10" t="s">
+      <c r="D4" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F4" s="25">
+      <c r="E4" s="26">
         <v>2000</v>
       </c>
-      <c r="K4" s="26" t="s">
+      <c r="J4" s="27" t="s">
         <v>46</v>
       </c>
-      <c r="L4" s="27">
+      <c r="K4" s="28">
         <v>1500</v>
       </c>
     </row>
-    <row r="5" spans="2:14">
-      <c r="C5" s="17" t="s">
+    <row r="5" spans="2:13">
+      <c r="B5" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="D5" s="25">
+      <c r="C5" s="11">
         <v>7500</v>
       </c>
-      <c r="E5" s="10" t="s">
+      <c r="D5" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="F5" s="25">
+      <c r="E5" s="26">
         <v>1000</v>
       </c>
       <c r="K5" s="17"/>
     </row>
-    <row r="6" spans="2:14">
+    <row r="6" spans="2:13">
       <c r="C6" s="17"/>
-      <c r="E6" s="10" t="s">
+      <c r="D6" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="F6" s="25">
+      <c r="E6" s="26">
         <v>3500</v>
       </c>
     </row>
-    <row r="7" spans="2:14">
+    <row r="7" spans="2:13">
       <c r="C7" s="17"/>
-      <c r="E7" s="10" t="s">
+      <c r="D7" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="F7" s="25">
+      <c r="E7" s="26">
         <v>2000</v>
       </c>
     </row>
-    <row r="8" spans="2:14">
+    <row r="8" spans="2:13">
       <c r="C8" s="17"/>
-      <c r="E8" s="10" t="s">
+      <c r="D8" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="F8" s="25">
+      <c r="E8" s="26">
         <v>3000</v>
       </c>
       <c r="K8" s="22" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="2:14">
-      <c r="C9" s="26" t="s">
+    <row r="9" spans="2:13">
+      <c r="B9" s="27" t="s">
         <v>46</v>
       </c>
-      <c r="D9" s="27">
+      <c r="C9" s="28">
         <v>45000</v>
       </c>
       <c r="J9" s="14"/>
@@ -1375,43 +1360,43 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="2:14">
+    <row r="10" spans="2:13">
       <c r="C10" s="17"/>
-      <c r="K10" s="17" t="s">
+      <c r="J10" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="L10" s="25">
+      <c r="K10" s="11">
         <v>6000</v>
       </c>
-      <c r="M10" s="10" t="s">
+      <c r="L10" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="N10" s="25">
+      <c r="M10" s="26">
         <v>4000</v>
       </c>
     </row>
-    <row r="11" spans="2:14">
+    <row r="11" spans="2:13">
       <c r="C11" s="17"/>
-      <c r="K11" s="26" t="s">
+      <c r="J11" s="27" t="s">
         <v>46</v>
       </c>
-      <c r="L11" s="27">
+      <c r="K11" s="28">
         <v>2000</v>
       </c>
     </row>
-    <row r="12" spans="2:14">
+    <row r="12" spans="2:13">
       <c r="C12" s="17"/>
       <c r="K12" s="17"/>
     </row>
-    <row r="17" spans="2:14">
+    <row r="17" spans="2:13">
       <c r="C17" s="22" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="K17" s="22" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="18" spans="2:14">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="18" spans="2:13">
       <c r="B18" s="14"/>
       <c r="C18" s="23" t="s">
         <v>3</v>
@@ -1429,48 +1414,48 @@
         <v>4</v>
       </c>
     </row>
-    <row r="19" spans="2:14">
+    <row r="19" spans="2:13">
       <c r="C19" s="8"/>
-      <c r="E19" s="10" t="s">
+      <c r="D19" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="F19" s="25">
+      <c r="E19" s="26">
         <v>50000</v>
       </c>
       <c r="K19" s="17"/>
-      <c r="M19" s="10" t="s">
+      <c r="L19" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="N19" s="25">
+      <c r="M19" s="26">
         <v>6000</v>
       </c>
     </row>
-    <row r="20" spans="2:14">
+    <row r="20" spans="2:13">
       <c r="C20" s="17"/>
-      <c r="E20" s="28" t="s">
+      <c r="D20" s="27" t="s">
         <v>46</v>
       </c>
-      <c r="F20" s="27">
+      <c r="E20" s="29">
         <v>50000</v>
       </c>
       <c r="K20" s="17"/>
-      <c r="M20" s="10" t="s">
+      <c r="L20" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="N20" s="25">
+      <c r="M20" s="26">
         <v>7500</v>
       </c>
     </row>
-    <row r="21" spans="2:14">
+    <row r="21" spans="2:13">
       <c r="K21" s="17"/>
-      <c r="M21" s="28" t="s">
+      <c r="L21" s="27" t="s">
         <v>46</v>
       </c>
-      <c r="N21" s="27">
+      <c r="M21" s="29">
         <v>13500</v>
       </c>
     </row>
-    <row r="26" spans="2:14">
+    <row r="26" spans="2:13">
       <c r="C26" s="22" t="s">
         <v>10</v>
       </c>
@@ -1478,7 +1463,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="27" spans="2:14">
+    <row r="27" spans="2:13">
       <c r="B27" s="14"/>
       <c r="C27" s="23" t="s">
         <v>3</v>
@@ -1496,46 +1481,46 @@
         <v>4</v>
       </c>
     </row>
-    <row r="28" spans="2:14">
-      <c r="C28" s="17" t="s">
+    <row r="28" spans="2:13">
+      <c r="B28" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="D28" s="25">
+      <c r="C28" s="11">
         <v>10000</v>
       </c>
-      <c r="K28" s="17" t="s">
+      <c r="J28" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="L28" s="25">
+      <c r="K28" s="11">
         <v>3500</v>
       </c>
     </row>
-    <row r="29" spans="2:14">
-      <c r="C29" s="17" t="s">
+    <row r="29" spans="2:13">
+      <c r="B29" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="D29" s="25">
+      <c r="C29" s="11">
         <v>1000</v>
       </c>
-      <c r="K29" s="26" t="s">
+      <c r="J29" s="27" t="s">
         <v>46</v>
       </c>
-      <c r="L29" s="27">
+      <c r="K29" s="28">
         <v>3500</v>
       </c>
     </row>
-    <row r="30" spans="2:14">
+    <row r="30" spans="2:13">
       <c r="C30" s="17"/>
       <c r="K30" s="17"/>
     </row>
-    <row r="31" spans="2:14">
+    <row r="31" spans="2:13">
       <c r="C31" s="17"/>
     </row>
     <row r="33" spans="2:13">
-      <c r="B33" s="28" t="s">
+      <c r="B33" s="27" t="s">
         <v>46</v>
       </c>
-      <c r="C33" s="27">
+      <c r="C33" s="29">
         <v>11000</v>
       </c>
     </row>
@@ -1566,75 +1551,74 @@
       </c>
     </row>
     <row r="37" spans="2:13">
-      <c r="C37" s="10" t="s">
+      <c r="B37" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="D37" s="29">
+      <c r="C37" s="26">
         <v>1000</v>
       </c>
-      <c r="E37" s="10" t="s">
+      <c r="D37" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="F37" s="25">
+      <c r="E37" s="26">
         <v>5000</v>
       </c>
-      <c r="K37" s="17" t="s">
+      <c r="J37" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="L37" s="25">
+      <c r="K37" s="11">
         <v>1200</v>
       </c>
     </row>
     <row r="38" spans="2:13">
-      <c r="C38" s="10" t="s">
+      <c r="B38" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="D38" s="29">
+      <c r="C38" s="26">
         <v>3000</v>
       </c>
-      <c r="E38" s="10" t="s">
+      <c r="D38" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="F38" s="25">
+      <c r="E38" s="26">
         <v>1500</v>
       </c>
-      <c r="K38" s="26" t="s">
+      <c r="J38" s="27" t="s">
         <v>46</v>
       </c>
-      <c r="L38" s="27">
+      <c r="K38" s="28">
         <v>1200</v>
       </c>
     </row>
     <row r="39" spans="2:13">
       <c r="C39" s="17"/>
-      <c r="E39" s="10" t="s">
+      <c r="D39" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="F39" s="25">
+      <c r="E39" s="26">
         <v>1200</v>
       </c>
       <c r="K39" s="17"/>
     </row>
     <row r="40" spans="2:13">
-      <c r="D40" s="30"/>
-      <c r="E40" s="10" t="s">
+      <c r="D40" s="30" t="s">
         <v>41</v>
       </c>
-      <c r="F40" s="25">
+      <c r="E40" s="26">
         <v>1000</v>
       </c>
     </row>
     <row r="41" spans="2:13">
-      <c r="E41" s="28" t="s">
+      <c r="D41" s="27" t="s">
         <v>46</v>
       </c>
-      <c r="F41" s="27">
+      <c r="E41" s="29">
         <v>4700</v>
       </c>
     </row>
     <row r="44" spans="2:13">
       <c r="C44" s="22" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="45" spans="2:13">
@@ -1648,18 +1632,19 @@
       </c>
     </row>
     <row r="46" spans="2:13">
-      <c r="C46" s="10" t="s">
+      <c r="B46" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="D46" s="29">
+      <c r="C46" s="26">
         <v>2000</v>
       </c>
+      <c r="D46" s="30"/>
     </row>
     <row r="47" spans="2:13">
-      <c r="C47" s="26" t="s">
+      <c r="B47" s="27" t="s">
         <v>46</v>
       </c>
-      <c r="D47" s="27">
+      <c r="C47" s="28">
         <v>2000</v>
       </c>
     </row>
@@ -1719,7 +1704,7 @@
     </row>
     <row r="75" spans="2:13">
       <c r="C75" s="22" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="76" spans="2:13">
@@ -1737,19 +1722,19 @@
       <c r="M76" s="14"/>
     </row>
     <row r="77" spans="2:13">
-      <c r="C77" s="8" t="s">
+      <c r="B77" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="D77" s="25">
+      <c r="C77" s="25">
         <v>2000</v>
       </c>
       <c r="K77" s="8"/>
     </row>
     <row r="78" spans="2:13">
-      <c r="C78" s="26" t="s">
+      <c r="B78" s="27" t="s">
         <v>46</v>
       </c>
-      <c r="D78" s="27">
+      <c r="C78" s="28">
         <v>2000</v>
       </c>
       <c r="K78" s="17"/>
@@ -1764,8 +1749,9 @@
   <dimension ref="A1:N25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="30.7109375" customWidth="1"/>
-    <col min="2" max="3" width="15.7109375" customWidth="1"/>
+    <col min="1" max="1" width="35.7109375" customWidth="1"/>
+    <col min="2" max="2" width="20.42578125" customWidth="1"/>
+    <col min="3" max="3" width="21.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1790,7 +1776,7 @@
       <c r="A3" s="30" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="29">
+      <c r="B3" s="33">
         <v>45000</v>
       </c>
       <c r="C3" s="9"/>
@@ -1799,7 +1785,7 @@
       <c r="A4" s="30" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="29">
+      <c r="B4" s="33">
         <v>2000</v>
       </c>
       <c r="C4" s="9"/>
@@ -1808,7 +1794,7 @@
       <c r="A5" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="29">
+      <c r="B5" s="33">
         <v>1500</v>
       </c>
       <c r="C5" s="9"/>
@@ -1817,7 +1803,7 @@
       <c r="A6" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="29">
+      <c r="B6" s="33">
         <v>11000</v>
       </c>
       <c r="C6" s="9"/>
@@ -1844,14 +1830,14 @@
       <c r="A9" s="30" t="s">
         <v>34</v>
       </c>
-      <c r="B9" s="29">
+      <c r="B9" s="33">
         <v>2000</v>
       </c>
       <c r="C9" s="9"/>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" s="30" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B10" s="30"/>
       <c r="C10" s="16">
@@ -1862,7 +1848,7 @@
       <c r="A11" s="30" t="s">
         <v>31</v>
       </c>
-      <c r="B11" s="29">
+      <c r="B11" s="33">
         <v>3500</v>
       </c>
       <c r="C11" s="9"/>
@@ -1871,7 +1857,7 @@
       <c r="A12" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="29">
+      <c r="B12" s="33">
         <v>2000</v>
       </c>
       <c r="C12" s="9"/>
@@ -1880,174 +1866,165 @@
       <c r="A13" s="30" t="s">
         <v>37</v>
       </c>
-      <c r="B13" s="29">
+      <c r="B13" s="33">
         <v>1200</v>
       </c>
       <c r="C13" s="9"/>
     </row>
     <row r="14" spans="1:3">
-      <c r="A14" s="33" t="s">
+      <c r="A14" s="34" t="s">
         <v>54</v>
       </c>
-      <c r="B14" s="34">
+      <c r="B14" s="35">
         <v>68200</v>
       </c>
-      <c r="C14" s="35">
+      <c r="C14" s="36">
         <v>68200</v>
       </c>
     </row>
-    <row r="15" spans="1:3">
-      <c r="A15" s="30"/>
-      <c r="B15" s="30"/>
-      <c r="C15" s="9"/>
-    </row>
     <row r="16" spans="1:3">
-      <c r="A16" s="28" t="s">
+      <c r="A16" s="27" t="s">
         <v>55</v>
       </c>
-      <c r="B16" s="30"/>
-      <c r="C16" s="9"/>
     </row>
     <row r="17" spans="1:14">
-      <c r="A17" s="36" t="s">
+      <c r="A17" s="37" t="s">
         <v>56</v>
       </c>
-      <c r="B17" s="36"/>
-      <c r="C17" s="36"/>
-      <c r="D17" s="36"/>
-      <c r="E17" s="36"/>
-      <c r="F17" s="36"/>
-      <c r="G17" s="36"/>
-      <c r="H17" s="36"/>
-      <c r="I17" s="36"/>
-      <c r="J17" s="36"/>
-      <c r="K17" s="36"/>
-      <c r="L17" s="36"/>
-      <c r="M17" s="36"/>
-      <c r="N17" s="36"/>
+      <c r="B17" s="37"/>
+      <c r="C17" s="37"/>
+      <c r="D17" s="37"/>
+      <c r="E17" s="37"/>
+      <c r="F17" s="37"/>
+      <c r="G17" s="37"/>
+      <c r="H17" s="37"/>
+      <c r="I17" s="37"/>
+      <c r="J17" s="37"/>
+      <c r="K17" s="37"/>
+      <c r="L17" s="37"/>
+      <c r="M17" s="37"/>
+      <c r="N17" s="37"/>
     </row>
     <row r="18" spans="1:14">
-      <c r="A18" s="36"/>
-      <c r="B18" s="36"/>
-      <c r="C18" s="36"/>
-      <c r="D18" s="36"/>
-      <c r="E18" s="36"/>
-      <c r="F18" s="36"/>
-      <c r="G18" s="36"/>
-      <c r="H18" s="36"/>
-      <c r="I18" s="36"/>
-      <c r="J18" s="36"/>
-      <c r="K18" s="36"/>
-      <c r="L18" s="36"/>
-      <c r="M18" s="36"/>
-      <c r="N18" s="36"/>
+      <c r="A18" s="37"/>
+      <c r="B18" s="37"/>
+      <c r="C18" s="37"/>
+      <c r="D18" s="37"/>
+      <c r="E18" s="37"/>
+      <c r="F18" s="37"/>
+      <c r="G18" s="37"/>
+      <c r="H18" s="37"/>
+      <c r="I18" s="37"/>
+      <c r="J18" s="37"/>
+      <c r="K18" s="37"/>
+      <c r="L18" s="37"/>
+      <c r="M18" s="37"/>
+      <c r="N18" s="37"/>
     </row>
     <row r="19" spans="1:14">
-      <c r="A19" s="36"/>
-      <c r="B19" s="36"/>
-      <c r="C19" s="36"/>
-      <c r="D19" s="36"/>
-      <c r="E19" s="36"/>
-      <c r="F19" s="36"/>
-      <c r="G19" s="36"/>
-      <c r="H19" s="36"/>
-      <c r="I19" s="36"/>
-      <c r="J19" s="36"/>
-      <c r="K19" s="36"/>
-      <c r="L19" s="36"/>
-      <c r="M19" s="36"/>
-      <c r="N19" s="36"/>
+      <c r="A19" s="37"/>
+      <c r="B19" s="37"/>
+      <c r="C19" s="37"/>
+      <c r="D19" s="37"/>
+      <c r="E19" s="37"/>
+      <c r="F19" s="37"/>
+      <c r="G19" s="37"/>
+      <c r="H19" s="37"/>
+      <c r="I19" s="37"/>
+      <c r="J19" s="37"/>
+      <c r="K19" s="37"/>
+      <c r="L19" s="37"/>
+      <c r="M19" s="37"/>
+      <c r="N19" s="37"/>
     </row>
     <row r="20" spans="1:14">
-      <c r="A20" s="36"/>
-      <c r="B20" s="36"/>
-      <c r="C20" s="36"/>
-      <c r="D20" s="36"/>
-      <c r="E20" s="36"/>
-      <c r="F20" s="36"/>
-      <c r="G20" s="36"/>
-      <c r="H20" s="36"/>
-      <c r="I20" s="36"/>
-      <c r="J20" s="36"/>
-      <c r="K20" s="36"/>
-      <c r="L20" s="36"/>
-      <c r="M20" s="36"/>
-      <c r="N20" s="36"/>
+      <c r="A20" s="37"/>
+      <c r="B20" s="37"/>
+      <c r="C20" s="37"/>
+      <c r="D20" s="37"/>
+      <c r="E20" s="37"/>
+      <c r="F20" s="37"/>
+      <c r="G20" s="37"/>
+      <c r="H20" s="37"/>
+      <c r="I20" s="37"/>
+      <c r="J20" s="37"/>
+      <c r="K20" s="37"/>
+      <c r="L20" s="37"/>
+      <c r="M20" s="37"/>
+      <c r="N20" s="37"/>
     </row>
     <row r="21" spans="1:14">
-      <c r="A21" s="36"/>
-      <c r="B21" s="36"/>
-      <c r="C21" s="36"/>
-      <c r="D21" s="36"/>
-      <c r="E21" s="36"/>
-      <c r="F21" s="36"/>
-      <c r="G21" s="36"/>
-      <c r="H21" s="36"/>
-      <c r="I21" s="36"/>
-      <c r="J21" s="36"/>
-      <c r="K21" s="36"/>
-      <c r="L21" s="36"/>
-      <c r="M21" s="36"/>
-      <c r="N21" s="36"/>
+      <c r="A21" s="37"/>
+      <c r="B21" s="37"/>
+      <c r="C21" s="37"/>
+      <c r="D21" s="37"/>
+      <c r="E21" s="37"/>
+      <c r="F21" s="37"/>
+      <c r="G21" s="37"/>
+      <c r="H21" s="37"/>
+      <c r="I21" s="37"/>
+      <c r="J21" s="37"/>
+      <c r="K21" s="37"/>
+      <c r="L21" s="37"/>
+      <c r="M21" s="37"/>
+      <c r="N21" s="37"/>
     </row>
     <row r="22" spans="1:14">
-      <c r="A22" s="28" t="s">
+      <c r="A22" s="27" t="s">
         <v>57</v>
       </c>
-      <c r="B22" s="37"/>
-      <c r="C22" s="38"/>
     </row>
     <row r="23" spans="1:14">
-      <c r="A23" s="36" t="s">
+      <c r="A23" s="37" t="s">
         <v>58</v>
       </c>
-      <c r="B23" s="36"/>
-      <c r="C23" s="36"/>
-      <c r="D23" s="36"/>
-      <c r="E23" s="36"/>
-      <c r="F23" s="36"/>
-      <c r="G23" s="36"/>
-      <c r="H23" s="36"/>
-      <c r="I23" s="36"/>
-      <c r="J23" s="36"/>
-      <c r="K23" s="36"/>
-      <c r="L23" s="36"/>
-      <c r="M23" s="36"/>
-      <c r="N23" s="36"/>
+      <c r="B23" s="37"/>
+      <c r="C23" s="37"/>
+      <c r="D23" s="37"/>
+      <c r="E23" s="37"/>
+      <c r="F23" s="37"/>
+      <c r="G23" s="37"/>
+      <c r="H23" s="37"/>
+      <c r="I23" s="37"/>
+      <c r="J23" s="37"/>
+      <c r="K23" s="37"/>
+      <c r="L23" s="37"/>
+      <c r="M23" s="37"/>
+      <c r="N23" s="37"/>
     </row>
     <row r="24" spans="1:14">
-      <c r="A24" s="36"/>
-      <c r="B24" s="36"/>
-      <c r="C24" s="36"/>
-      <c r="D24" s="36"/>
-      <c r="E24" s="36"/>
-      <c r="F24" s="36"/>
-      <c r="G24" s="36"/>
-      <c r="H24" s="36"/>
-      <c r="I24" s="36"/>
-      <c r="J24" s="36"/>
-      <c r="K24" s="36"/>
-      <c r="L24" s="36"/>
-      <c r="M24" s="36"/>
-      <c r="N24" s="36"/>
+      <c r="A24" s="37"/>
+      <c r="B24" s="37"/>
+      <c r="C24" s="37"/>
+      <c r="D24" s="37"/>
+      <c r="E24" s="37"/>
+      <c r="F24" s="37"/>
+      <c r="G24" s="37"/>
+      <c r="H24" s="37"/>
+      <c r="I24" s="37"/>
+      <c r="J24" s="37"/>
+      <c r="K24" s="37"/>
+      <c r="L24" s="37"/>
+      <c r="M24" s="37"/>
+      <c r="N24" s="37"/>
     </row>
     <row r="25" spans="1:14">
-      <c r="A25" s="39" t="s">
+      <c r="A25" s="38" t="s">
         <v>59</v>
       </c>
-      <c r="B25" s="36"/>
-      <c r="C25" s="36"/>
-      <c r="D25" s="36"/>
-      <c r="E25" s="36"/>
-      <c r="F25" s="36"/>
-      <c r="G25" s="36"/>
-      <c r="H25" s="36"/>
-      <c r="I25" s="36"/>
-      <c r="J25" s="36"/>
-      <c r="K25" s="36"/>
-      <c r="L25" s="36"/>
-      <c r="M25" s="36"/>
-      <c r="N25" s="36"/>
+      <c r="B25" s="37"/>
+      <c r="C25" s="37"/>
+      <c r="D25" s="37"/>
+      <c r="E25" s="37"/>
+      <c r="F25" s="37"/>
+      <c r="G25" s="37"/>
+      <c r="H25" s="37"/>
+      <c r="I25" s="37"/>
+      <c r="J25" s="37"/>
+      <c r="K25" s="37"/>
+      <c r="L25" s="37"/>
+      <c r="M25" s="37"/>
+      <c r="N25" s="37"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>